<commit_message>
feat(plot): Update outcomes and improve test coverage for forest and dot plots
</commit_message>
<xml_diff>
--- a/data-raw/Manuscript_Generic_Example.xlsx
+++ b/data-raw/Manuscript_Generic_Example.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25601"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28730"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\e618345\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lgaka\Downloads\brpubVJCE\data-raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED5B20D8-EF1C-4929-8CE3-46F9CF95FA10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45E440DB-7E6D-4DAC-9237-F4DD7BC63BA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Example Effects Table" sheetId="1" r:id="rId1"/>
@@ -578,24 +578,9 @@
     <t xml:space="preserve"> </t>
   </si>
   <si>
-    <t>Primary Efficacy</t>
-  </si>
-  <si>
-    <t>Secondary Efficacy</t>
-  </si>
-  <si>
-    <t>Rare SAE</t>
-  </si>
-  <si>
     <t>Toxicity</t>
   </si>
   <si>
-    <t>Liver</t>
-  </si>
-  <si>
-    <t>Reoccurring AE</t>
-  </si>
-  <si>
     <t>% Achieving Remission</t>
   </si>
   <si>
@@ -605,9 +590,6 @@
     <t>Incidence Rate</t>
   </si>
   <si>
-    <t>HR Quality of Life</t>
-  </si>
-  <si>
     <t>Comorbidities</t>
   </si>
   <si>
@@ -651,6 +633,24 @@
   </si>
   <si>
     <t>Drug D</t>
+  </si>
+  <si>
+    <t>Benefit 1</t>
+  </si>
+  <si>
+    <t>Benefit 2</t>
+  </si>
+  <si>
+    <t>Benefit 3</t>
+  </si>
+  <si>
+    <t>Risk 1</t>
+  </si>
+  <si>
+    <t>Risk 2</t>
+  </si>
+  <si>
+    <t>Risk 3</t>
   </si>
 </sst>
 </file>
@@ -660,7 +660,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.000"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -694,6 +694,12 @@
     <font>
       <sz val="12"/>
       <color rgb="FF333333"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -812,7 +818,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -888,7 +894,6 @@
     <xf numFmtId="164" fontId="0" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1170,24 +1175,24 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AY25"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="22.140625" customWidth="1"/>
-    <col min="3" max="3" width="20.85546875" customWidth="1"/>
-    <col min="4" max="4" width="26.42578125" customWidth="1"/>
-    <col min="5" max="5" width="14.7109375" customWidth="1"/>
-    <col min="6" max="6" width="10.5703125" customWidth="1"/>
-    <col min="7" max="7" width="12.28515625" customWidth="1"/>
-    <col min="15" max="15" width="9.140625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.1796875" customWidth="1"/>
+    <col min="3" max="3" width="20.81640625" customWidth="1"/>
+    <col min="4" max="4" width="26.453125" customWidth="1"/>
+    <col min="5" max="5" width="14.7265625" customWidth="1"/>
+    <col min="6" max="6" width="10.54296875" customWidth="1"/>
+    <col min="7" max="7" width="12.26953125" customWidth="1"/>
+    <col min="15" max="15" width="9.1796875" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="11.81640625" bestFit="1" customWidth="1"/>
     <col min="22" max="22" width="12" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="10.28515625" customWidth="1"/>
-    <col min="24" max="24" width="9.140625" customWidth="1"/>
-    <col min="29" max="29" width="9.140625" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="10.26953125" customWidth="1"/>
+    <col min="24" max="24" width="9.1796875" customWidth="1"/>
+    <col min="29" max="29" width="9.1796875" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="11.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:51" s="23" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:51" s="23" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="24" t="s">
         <v>0</v>
       </c>
@@ -1342,7 +1347,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="2" spans="1:51" s="23" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:51" s="23" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="23" t="s">
         <v>49</v>
       </c>
@@ -1350,10 +1355,10 @@
         <v>50</v>
       </c>
       <c r="C2" s="23" t="s">
-        <v>175</v>
+        <v>194</v>
       </c>
       <c r="D2" s="23" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="E2" s="23" t="s">
         <v>51</v>
@@ -1368,7 +1373,7 @@
         <v>54</v>
       </c>
       <c r="J2" s="29" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="K2" s="23">
         <v>300</v>
@@ -1418,7 +1423,7 @@
       <c r="AI2" s="33"/>
       <c r="AJ2" s="33"/>
     </row>
-    <row r="3" spans="1:51" s="23" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:51" s="23" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A3" s="23" t="s">
         <v>49</v>
       </c>
@@ -1426,7 +1431,7 @@
         <v>50</v>
       </c>
       <c r="C3" s="23" t="s">
-        <v>176</v>
+        <v>195</v>
       </c>
       <c r="D3" s="23" t="s">
         <v>58</v>
@@ -1444,7 +1449,7 @@
         <v>54</v>
       </c>
       <c r="J3" s="29" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="K3" s="33"/>
       <c r="L3" s="23">
@@ -1490,7 +1495,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:51" s="23" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:51" s="23" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A4" s="23" t="s">
         <v>49</v>
       </c>
@@ -1498,7 +1503,7 @@
         <v>57</v>
       </c>
       <c r="C4" s="23" t="s">
-        <v>184</v>
+        <v>196</v>
       </c>
       <c r="D4" s="23" t="s">
         <v>58</v>
@@ -1516,7 +1521,7 @@
         <v>54</v>
       </c>
       <c r="J4" s="29" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="K4" s="33"/>
       <c r="L4" s="23">
@@ -1559,7 +1564,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:51" s="23" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:51" s="23" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A5" s="23" t="s">
         <v>61</v>
       </c>
@@ -1567,10 +1572,10 @@
         <v>62</v>
       </c>
       <c r="C5" s="23" t="s">
-        <v>180</v>
+        <v>197</v>
       </c>
       <c r="D5" s="23" t="s">
-        <v>182</v>
+        <v>177</v>
       </c>
       <c r="E5" s="23" t="s">
         <v>51</v>
@@ -1588,7 +1593,7 @@
         <v>54</v>
       </c>
       <c r="J5" s="29" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="K5" s="23">
         <v>300</v>
@@ -1651,7 +1656,7 @@
       <c r="AI5" s="33"/>
       <c r="AJ5" s="33"/>
     </row>
-    <row r="6" spans="1:51" s="23" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:51" s="23" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A6" s="23" t="s">
         <v>61</v>
       </c>
@@ -1659,10 +1664,10 @@
         <v>62</v>
       </c>
       <c r="C6" s="23" t="s">
-        <v>177</v>
+        <v>198</v>
       </c>
       <c r="D6" s="23" t="s">
-        <v>183</v>
+        <v>178</v>
       </c>
       <c r="E6" s="23" t="s">
         <v>51</v>
@@ -1680,7 +1685,7 @@
         <v>54</v>
       </c>
       <c r="J6" s="29" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="K6" s="23">
         <v>15</v>
@@ -1740,18 +1745,18 @@
       <c r="AI6" s="33"/>
       <c r="AJ6" s="33"/>
     </row>
-    <row r="7" spans="1:51" s="23" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:51" s="23" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A7" s="23" t="s">
         <v>61</v>
       </c>
       <c r="B7" s="23" t="s">
+        <v>175</v>
+      </c>
+      <c r="C7" s="23" t="s">
+        <v>199</v>
+      </c>
+      <c r="D7" s="23" t="s">
         <v>178</v>
-      </c>
-      <c r="C7" s="23" t="s">
-        <v>179</v>
-      </c>
-      <c r="D7" s="23" t="s">
-        <v>183</v>
       </c>
       <c r="E7" s="23" t="s">
         <v>51</v>
@@ -1769,7 +1774,7 @@
         <v>54</v>
       </c>
       <c r="J7" s="29" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="K7" s="23">
         <v>4</v>
@@ -1830,7 +1835,7 @@
       <c r="AI7" s="33"/>
       <c r="AJ7" s="33"/>
     </row>
-    <row r="8" spans="1:51" s="30" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:51" s="30" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A8" s="30" t="s">
         <v>49</v>
       </c>
@@ -1838,10 +1843,10 @@
         <v>50</v>
       </c>
       <c r="C8" s="30" t="s">
-        <v>175</v>
+        <v>194</v>
       </c>
       <c r="D8" s="30" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="E8" s="30" t="s">
         <v>51</v>
@@ -1856,7 +1861,7 @@
         <v>54</v>
       </c>
       <c r="J8" s="30" t="s">
-        <v>197</v>
+        <v>191</v>
       </c>
       <c r="K8" s="30">
         <v>175</v>
@@ -1906,7 +1911,7 @@
       <c r="AI8" s="33"/>
       <c r="AJ8" s="33"/>
     </row>
-    <row r="9" spans="1:51" s="30" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:51" s="30" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A9" s="30" t="s">
         <v>49</v>
       </c>
@@ -1914,7 +1919,7 @@
         <v>50</v>
       </c>
       <c r="C9" s="30" t="s">
-        <v>176</v>
+        <v>195</v>
       </c>
       <c r="D9" s="23" t="s">
         <v>58</v>
@@ -1932,7 +1937,7 @@
         <v>54</v>
       </c>
       <c r="J9" s="30" t="s">
-        <v>197</v>
+        <v>191</v>
       </c>
       <c r="L9" s="30">
         <v>1000</v>
@@ -1975,7 +1980,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="10" spans="1:51" s="30" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:51" s="30" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A10" s="30" t="s">
         <v>49</v>
       </c>
@@ -1983,7 +1988,7 @@
         <v>57</v>
       </c>
       <c r="C10" s="30" t="s">
-        <v>184</v>
+        <v>196</v>
       </c>
       <c r="D10" s="30" t="s">
         <v>58</v>
@@ -2001,7 +2006,7 @@
         <v>54</v>
       </c>
       <c r="J10" s="30" t="s">
-        <v>197</v>
+        <v>191</v>
       </c>
       <c r="K10" s="33"/>
       <c r="L10" s="30">
@@ -2019,7 +2024,7 @@
       <c r="T10" s="30">
         <v>58</v>
       </c>
-      <c r="V10" s="41">
+      <c r="V10" s="30">
         <v>58</v>
       </c>
       <c r="W10" s="30" t="s">
@@ -2046,7 +2051,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="11" spans="1:51" s="30" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:51" s="30" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A11" s="30" t="s">
         <v>61</v>
       </c>
@@ -2054,10 +2059,10 @@
         <v>62</v>
       </c>
       <c r="C11" s="30" t="s">
-        <v>180</v>
+        <v>197</v>
       </c>
       <c r="D11" s="30" t="s">
-        <v>182</v>
+        <v>177</v>
       </c>
       <c r="E11" s="30" t="s">
         <v>51</v>
@@ -2075,7 +2080,7 @@
         <v>54</v>
       </c>
       <c r="J11" s="30" t="s">
-        <v>197</v>
+        <v>191</v>
       </c>
       <c r="K11" s="30">
         <v>300</v>
@@ -2138,7 +2143,7 @@
       <c r="AI11" s="33"/>
       <c r="AJ11" s="33"/>
     </row>
-    <row r="12" spans="1:51" s="30" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:51" s="30" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A12" s="30" t="s">
         <v>61</v>
       </c>
@@ -2146,10 +2151,10 @@
         <v>62</v>
       </c>
       <c r="C12" s="30" t="s">
-        <v>177</v>
+        <v>198</v>
       </c>
       <c r="D12" s="30" t="s">
-        <v>183</v>
+        <v>178</v>
       </c>
       <c r="E12" s="30" t="s">
         <v>51</v>
@@ -2167,7 +2172,7 @@
         <v>54</v>
       </c>
       <c r="J12" s="30" t="s">
-        <v>197</v>
+        <v>191</v>
       </c>
       <c r="K12" s="30">
         <v>10</v>
@@ -2228,18 +2233,18 @@
       <c r="AI12" s="33"/>
       <c r="AJ12" s="33"/>
     </row>
-    <row r="13" spans="1:51" s="30" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:51" s="30" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A13" s="30" t="s">
         <v>61</v>
       </c>
       <c r="B13" s="30" t="s">
+        <v>175</v>
+      </c>
+      <c r="C13" s="30" t="s">
+        <v>198</v>
+      </c>
+      <c r="D13" s="30" t="s">
         <v>178</v>
-      </c>
-      <c r="C13" s="30" t="s">
-        <v>179</v>
-      </c>
-      <c r="D13" s="30" t="s">
-        <v>183</v>
       </c>
       <c r="E13" s="30" t="s">
         <v>51</v>
@@ -2257,7 +2262,7 @@
         <v>54</v>
       </c>
       <c r="J13" s="30" t="s">
-        <v>197</v>
+        <v>191</v>
       </c>
       <c r="K13" s="30">
         <v>2</v>
@@ -2318,7 +2323,7 @@
       <c r="AI13" s="33"/>
       <c r="AJ13" s="33"/>
     </row>
-    <row r="14" spans="1:51" s="31" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:51" s="31" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A14" s="31" t="s">
         <v>49</v>
       </c>
@@ -2326,10 +2331,10 @@
         <v>50</v>
       </c>
       <c r="C14" s="31" t="s">
-        <v>175</v>
+        <v>194</v>
       </c>
       <c r="D14" s="31" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="E14" s="31" t="s">
         <v>51</v>
@@ -2344,7 +2349,7 @@
         <v>54</v>
       </c>
       <c r="J14" s="31" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
       <c r="K14" s="31">
         <v>200</v>
@@ -2394,7 +2399,7 @@
       <c r="AI14" s="33"/>
       <c r="AJ14" s="33"/>
     </row>
-    <row r="15" spans="1:51" s="31" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:51" s="31" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A15" s="31" t="s">
         <v>49</v>
       </c>
@@ -2402,7 +2407,7 @@
         <v>50</v>
       </c>
       <c r="C15" s="31" t="s">
-        <v>176</v>
+        <v>195</v>
       </c>
       <c r="D15" s="23" t="s">
         <v>58</v>
@@ -2420,7 +2425,7 @@
         <v>54</v>
       </c>
       <c r="J15" s="31" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
       <c r="L15" s="31">
         <v>1000</v>
@@ -2463,7 +2468,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="16" spans="1:51" s="31" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:51" s="31" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A16" s="31" t="s">
         <v>49</v>
       </c>
@@ -2471,7 +2476,7 @@
         <v>57</v>
       </c>
       <c r="C16" s="31" t="s">
-        <v>184</v>
+        <v>196</v>
       </c>
       <c r="D16" s="31" t="s">
         <v>58</v>
@@ -2489,7 +2494,7 @@
         <v>54</v>
       </c>
       <c r="J16" s="31" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
       <c r="K16" s="33"/>
       <c r="L16" s="31">
@@ -2534,7 +2539,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="17" spans="1:36" s="31" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:36" s="31" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A17" s="31" t="s">
         <v>61</v>
       </c>
@@ -2542,10 +2547,10 @@
         <v>62</v>
       </c>
       <c r="C17" s="31" t="s">
-        <v>180</v>
+        <v>197</v>
       </c>
       <c r="D17" s="31" t="s">
-        <v>182</v>
+        <v>177</v>
       </c>
       <c r="E17" s="31" t="s">
         <v>51</v>
@@ -2563,7 +2568,7 @@
         <v>54</v>
       </c>
       <c r="J17" s="31" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
       <c r="K17" s="31">
         <v>300</v>
@@ -2626,7 +2631,7 @@
       <c r="AI17" s="33"/>
       <c r="AJ17" s="33"/>
     </row>
-    <row r="18" spans="1:36" s="31" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:36" s="31" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A18" s="31" t="s">
         <v>61</v>
       </c>
@@ -2634,10 +2639,10 @@
         <v>62</v>
       </c>
       <c r="C18" s="31" t="s">
-        <v>177</v>
+        <v>198</v>
       </c>
       <c r="D18" s="31" t="s">
-        <v>183</v>
+        <v>178</v>
       </c>
       <c r="E18" s="31" t="s">
         <v>51</v>
@@ -2655,7 +2660,7 @@
         <v>54</v>
       </c>
       <c r="J18" s="31" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
       <c r="K18" s="31">
         <v>20</v>
@@ -2716,18 +2721,18 @@
       <c r="AI18" s="33"/>
       <c r="AJ18" s="33"/>
     </row>
-    <row r="19" spans="1:36" s="31" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:36" s="31" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A19" s="31" t="s">
         <v>61</v>
       </c>
       <c r="B19" s="31" t="s">
+        <v>175</v>
+      </c>
+      <c r="C19" s="31" t="s">
+        <v>199</v>
+      </c>
+      <c r="D19" s="31" t="s">
         <v>178</v>
-      </c>
-      <c r="C19" s="31" t="s">
-        <v>179</v>
-      </c>
-      <c r="D19" s="31" t="s">
-        <v>183</v>
       </c>
       <c r="E19" s="31" t="s">
         <v>51</v>
@@ -2745,7 +2750,7 @@
         <v>54</v>
       </c>
       <c r="J19" s="31" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
       <c r="K19" s="31">
         <v>6</v>
@@ -2806,7 +2811,7 @@
       <c r="AI19" s="33"/>
       <c r="AJ19" s="33"/>
     </row>
-    <row r="20" spans="1:36" s="32" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:36" s="32" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A20" s="32" t="s">
         <v>49</v>
       </c>
@@ -2814,10 +2819,10 @@
         <v>50</v>
       </c>
       <c r="C20" s="32" t="s">
-        <v>175</v>
+        <v>194</v>
       </c>
       <c r="D20" s="32" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="E20" s="32" t="s">
         <v>51</v>
@@ -2832,7 +2837,7 @@
         <v>54</v>
       </c>
       <c r="J20" s="32" t="s">
-        <v>199</v>
+        <v>193</v>
       </c>
       <c r="K20" s="32">
         <v>100</v>
@@ -2882,7 +2887,7 @@
       <c r="AI20" s="33"/>
       <c r="AJ20" s="33"/>
     </row>
-    <row r="21" spans="1:36" s="32" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:36" s="32" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A21" s="32" t="s">
         <v>49</v>
       </c>
@@ -2890,7 +2895,7 @@
         <v>50</v>
       </c>
       <c r="C21" s="32" t="s">
-        <v>176</v>
+        <v>195</v>
       </c>
       <c r="D21" s="23" t="s">
         <v>58</v>
@@ -2908,7 +2913,7 @@
         <v>54</v>
       </c>
       <c r="J21" s="32" t="s">
-        <v>199</v>
+        <v>193</v>
       </c>
       <c r="L21" s="32">
         <v>1000</v>
@@ -2961,7 +2966,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="22" spans="1:36" s="32" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:36" s="32" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A22" s="32" t="s">
         <v>49</v>
       </c>
@@ -2969,7 +2974,7 @@
         <v>57</v>
       </c>
       <c r="C22" s="32" t="s">
-        <v>184</v>
+        <v>196</v>
       </c>
       <c r="D22" s="32" t="s">
         <v>58</v>
@@ -2987,7 +2992,7 @@
         <v>54</v>
       </c>
       <c r="J22" s="32" t="s">
-        <v>199</v>
+        <v>193</v>
       </c>
       <c r="K22" s="33"/>
       <c r="L22" s="32">
@@ -3033,7 +3038,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="23" spans="1:36" s="32" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:36" s="32" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A23" s="32" t="s">
         <v>61</v>
       </c>
@@ -3041,10 +3046,10 @@
         <v>62</v>
       </c>
       <c r="C23" s="32" t="s">
-        <v>180</v>
+        <v>197</v>
       </c>
       <c r="D23" s="32" t="s">
-        <v>182</v>
+        <v>177</v>
       </c>
       <c r="E23" s="32" t="s">
         <v>51</v>
@@ -3062,7 +3067,7 @@
         <v>54</v>
       </c>
       <c r="J23" s="32" t="s">
-        <v>199</v>
+        <v>193</v>
       </c>
       <c r="K23" s="32">
         <v>80</v>
@@ -3126,7 +3131,7 @@
       <c r="AI23" s="33"/>
       <c r="AJ23" s="33"/>
     </row>
-    <row r="24" spans="1:36" s="32" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:36" s="32" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A24" s="32" t="s">
         <v>61</v>
       </c>
@@ -3134,10 +3139,10 @@
         <v>62</v>
       </c>
       <c r="C24" s="32" t="s">
-        <v>177</v>
+        <v>198</v>
       </c>
       <c r="D24" s="32" t="s">
-        <v>183</v>
+        <v>178</v>
       </c>
       <c r="E24" s="32" t="s">
         <v>51</v>
@@ -3155,7 +3160,7 @@
         <v>54</v>
       </c>
       <c r="J24" s="32" t="s">
-        <v>199</v>
+        <v>193</v>
       </c>
       <c r="K24" s="32">
         <v>12</v>
@@ -3216,18 +3221,18 @@
       <c r="AI24" s="33"/>
       <c r="AJ24" s="33"/>
     </row>
-    <row r="25" spans="1:36" s="32" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:36" s="32" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A25" s="32" t="s">
         <v>61</v>
       </c>
       <c r="B25" s="32" t="s">
+        <v>175</v>
+      </c>
+      <c r="C25" s="32" t="s">
+        <v>199</v>
+      </c>
+      <c r="D25" s="32" t="s">
         <v>178</v>
-      </c>
-      <c r="C25" s="32" t="s">
-        <v>179</v>
-      </c>
-      <c r="D25" s="32" t="s">
-        <v>183</v>
       </c>
       <c r="E25" s="32" t="s">
         <v>51</v>
@@ -3245,7 +3250,7 @@
         <v>54</v>
       </c>
       <c r="J25" s="32" t="s">
-        <v>199</v>
+        <v>193</v>
       </c>
       <c r="K25" s="32">
         <v>0</v>
@@ -3307,7 +3312,7 @@
       <c r="AJ25" s="33"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AY25" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
@@ -3316,184 +3321,184 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5D4A282F-FA68-4BC3-9814-08A63A8C35E3}">
   <dimension ref="A1:C16"/>
-  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="16.42578125" style="16" customWidth="1"/>
-    <col min="2" max="2" width="7.140625" style="16" customWidth="1"/>
-    <col min="3" max="3" width="12.28515625" style="17" customWidth="1"/>
+    <col min="1" max="1" width="16.453125" style="16" customWidth="1"/>
+    <col min="2" max="2" width="7.1796875" style="16" customWidth="1"/>
+    <col min="3" max="3" width="12.26953125" style="17" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" s="15" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" s="15" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="18" t="s">
-        <v>185</v>
+        <v>179</v>
       </c>
       <c r="B1" s="18" t="s">
-        <v>195</v>
+        <v>189</v>
       </c>
       <c r="C1" s="19" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" s="20" t="s">
+        <v>182</v>
+      </c>
+      <c r="B2" s="20" t="s">
         <v>186</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" s="20" t="s">
-        <v>188</v>
-      </c>
-      <c r="B2" s="20" t="s">
-        <v>192</v>
       </c>
       <c r="C2" s="21">
         <v>0.02</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" s="20" t="s">
-        <v>188</v>
+        <v>182</v>
       </c>
       <c r="B3" s="20" t="s">
-        <v>193</v>
+        <v>187</v>
       </c>
       <c r="C3" s="21">
         <v>0.12</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" s="20" t="s">
+        <v>182</v>
+      </c>
+      <c r="B4" s="20" t="s">
         <v>188</v>
-      </c>
-      <c r="B4" s="20" t="s">
-        <v>194</v>
       </c>
       <c r="C4" s="21">
         <v>0.25</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" s="20" t="s">
-        <v>187</v>
+        <v>181</v>
       </c>
       <c r="B5" s="20" t="s">
-        <v>192</v>
+        <v>186</v>
       </c>
       <c r="C5" s="21">
         <v>0.01</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" s="20" t="s">
+        <v>181</v>
+      </c>
+      <c r="B6" s="20" t="s">
         <v>187</v>
-      </c>
-      <c r="B6" s="20" t="s">
-        <v>193</v>
       </c>
       <c r="C6" s="21">
         <v>0.1</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" s="20" t="s">
-        <v>187</v>
+        <v>181</v>
       </c>
       <c r="B7" s="20" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="C7" s="21">
         <v>0.15</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" s="20" t="s">
-        <v>189</v>
+        <v>183</v>
       </c>
       <c r="B8" s="20" t="s">
-        <v>192</v>
+        <v>186</v>
       </c>
       <c r="C8" s="21">
         <v>0.05</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" s="20" t="s">
-        <v>189</v>
+        <v>183</v>
       </c>
       <c r="B9" s="20" t="s">
-        <v>193</v>
+        <v>187</v>
       </c>
       <c r="C9" s="21">
         <v>0.25</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10" s="20" t="s">
-        <v>189</v>
+        <v>183</v>
       </c>
       <c r="B10" s="20" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="C10" s="21">
         <v>0.4</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A11" s="22" t="s">
-        <v>190</v>
+        <v>184</v>
       </c>
       <c r="B11" s="20" t="s">
-        <v>192</v>
+        <v>186</v>
       </c>
       <c r="C11" s="21">
         <v>1E-3</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A12" s="20" t="s">
-        <v>190</v>
+        <v>184</v>
       </c>
       <c r="B12" s="20" t="s">
-        <v>193</v>
+        <v>187</v>
       </c>
       <c r="C12" s="21">
         <v>0.12</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A13" s="20" t="s">
-        <v>190</v>
+        <v>184</v>
       </c>
       <c r="B13" s="20" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="C13" s="21">
         <v>0.2</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A14" s="20" t="s">
-        <v>191</v>
+        <v>185</v>
       </c>
       <c r="B14" s="20" t="s">
-        <v>192</v>
+        <v>186</v>
       </c>
       <c r="C14" s="21">
         <v>1E-3</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A15" s="20" t="s">
-        <v>191</v>
+        <v>185</v>
       </c>
       <c r="B15" s="20" t="s">
-        <v>193</v>
+        <v>187</v>
       </c>
       <c r="C15" s="21">
         <v>0.05</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A16" s="20" t="s">
-        <v>191</v>
+        <v>185</v>
       </c>
       <c r="B16" s="20" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="C16" s="21">
         <v>0.15</v>
@@ -3507,18 +3512,18 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F7B77BDC-7246-43E5-B2E5-9DD908E43155}">
   <dimension ref="A1:G60"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="17.42578125" style="13" customWidth="1"/>
-    <col min="2" max="2" width="21.85546875" style="13" customWidth="1"/>
-    <col min="3" max="3" width="42.5703125" style="13" customWidth="1"/>
-    <col min="4" max="4" width="9.7109375" style="14" customWidth="1"/>
+    <col min="1" max="1" width="17.453125" style="13" customWidth="1"/>
+    <col min="2" max="2" width="21.81640625" style="13" customWidth="1"/>
+    <col min="3" max="3" width="42.54296875" style="13" customWidth="1"/>
+    <col min="4" max="4" width="9.7265625" style="14" customWidth="1"/>
     <col min="5" max="5" width="18" style="13" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="22.5703125" style="13" customWidth="1"/>
-    <col min="7" max="7" width="35.28515625" style="14" customWidth="1"/>
+    <col min="6" max="6" width="22.54296875" style="13" customWidth="1"/>
+    <col min="7" max="7" width="35.26953125" style="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" s="1" customFormat="1" ht="120" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" s="1" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>170</v>
       </c>
@@ -3541,7 +3546,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
         <v>0</v>
       </c>
@@ -3560,7 +3565,7 @@
       <c r="F2" s="3"/>
       <c r="G2" s="4"/>
     </row>
-    <row r="3" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
@@ -3579,7 +3584,7 @@
       </c>
       <c r="G3" s="4"/>
     </row>
-    <row r="4" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -3598,7 +3603,7 @@
       </c>
       <c r="G4" s="4"/>
     </row>
-    <row r="5" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
         <v>3</v>
       </c>
@@ -3617,7 +3622,7 @@
       </c>
       <c r="G5" s="4"/>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
         <v>4</v>
       </c>
@@ -3636,7 +3641,7 @@
       <c r="F6" s="3"/>
       <c r="G6" s="4"/>
     </row>
-    <row r="7" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
         <v>6</v>
       </c>
@@ -3655,7 +3660,7 @@
       <c r="F7" s="3"/>
       <c r="G7" s="4"/>
     </row>
-    <row r="8" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
         <v>7</v>
       </c>
@@ -3676,7 +3681,7 @@
       </c>
       <c r="G8" s="4"/>
     </row>
-    <row r="9" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
         <v>8</v>
       </c>
@@ -3697,7 +3702,7 @@
       </c>
       <c r="G9" s="4"/>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
         <v>9</v>
       </c>
@@ -3716,7 +3721,7 @@
       </c>
       <c r="G10" s="4"/>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
         <v>23</v>
       </c>
@@ -3735,7 +3740,7 @@
       <c r="F11" s="3"/>
       <c r="G11" s="4"/>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
         <v>22</v>
       </c>
@@ -3754,7 +3759,7 @@
       <c r="F12" s="3"/>
       <c r="G12" s="4"/>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A13" s="3"/>
       <c r="B13" s="3"/>
       <c r="C13" s="3"/>
@@ -3763,7 +3768,7 @@
       <c r="F13" s="3"/>
       <c r="G13" s="4"/>
     </row>
-    <row r="14" spans="1:7" ht="105" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A14" s="5" t="s">
         <v>169</v>
       </c>
@@ -3786,7 +3791,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="15" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A15" s="3" t="s">
         <v>5</v>
       </c>
@@ -3805,7 +3810,7 @@
       <c r="F15" s="3"/>
       <c r="G15" s="4"/>
     </row>
-    <row r="16" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A16" s="3" t="s">
         <v>12</v>
       </c>
@@ -3822,7 +3827,7 @@
       <c r="F16" s="3"/>
       <c r="G16" s="4"/>
     </row>
-    <row r="17" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" ht="58" x14ac:dyDescent="0.35">
       <c r="A17" s="3" t="s">
         <v>15</v>
       </c>
@@ -3839,7 +3844,7 @@
       <c r="F17" s="3"/>
       <c r="G17" s="4"/>
     </row>
-    <row r="18" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" ht="58" x14ac:dyDescent="0.35">
       <c r="A18" s="3" t="s">
         <v>18</v>
       </c>
@@ -3856,7 +3861,7 @@
       <c r="F18" s="3"/>
       <c r="G18" s="4"/>
     </row>
-    <row r="19" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A19" s="3" t="s">
         <v>19</v>
       </c>
@@ -3873,7 +3878,7 @@
       <c r="F19" s="3"/>
       <c r="G19" s="4"/>
     </row>
-    <row r="20" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A20" s="3" t="s">
         <v>26</v>
       </c>
@@ -3890,7 +3895,7 @@
       <c r="F20" s="3"/>
       <c r="G20" s="4"/>
     </row>
-    <row r="21" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" ht="58" x14ac:dyDescent="0.35">
       <c r="A21" s="3" t="s">
         <v>29</v>
       </c>
@@ -3907,7 +3912,7 @@
       <c r="F21" s="3"/>
       <c r="G21" s="4"/>
     </row>
-    <row r="22" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" ht="58" x14ac:dyDescent="0.35">
       <c r="A22" s="3" t="s">
         <v>32</v>
       </c>
@@ -3924,7 +3929,7 @@
       <c r="F22" s="3"/>
       <c r="G22" s="4"/>
     </row>
-    <row r="23" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A23" s="3" t="s">
         <v>33</v>
       </c>
@@ -3941,7 +3946,7 @@
       <c r="F23" s="3"/>
       <c r="G23" s="4"/>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A24" s="3"/>
       <c r="B24" s="3"/>
       <c r="C24" s="3"/>
@@ -3950,7 +3955,7 @@
       <c r="F24" s="3"/>
       <c r="G24" s="4"/>
     </row>
-    <row r="25" spans="1:7" ht="105" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7" ht="87" x14ac:dyDescent="0.35">
       <c r="A25" s="7" t="s">
         <v>171</v>
       </c>
@@ -3973,7 +3978,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="26" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A26" s="3" t="s">
         <v>11</v>
       </c>
@@ -3990,7 +3995,7 @@
       <c r="F26" s="3"/>
       <c r="G26" s="4"/>
     </row>
-    <row r="27" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A27" s="3" t="s">
         <v>14</v>
       </c>
@@ -4007,7 +4012,7 @@
       <c r="F27" s="3"/>
       <c r="G27" s="4"/>
     </row>
-    <row r="28" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A28" s="3" t="s">
         <v>17</v>
       </c>
@@ -4024,7 +4029,7 @@
       <c r="F28" s="3"/>
       <c r="G28" s="4"/>
     </row>
-    <row r="29" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:7" ht="58" x14ac:dyDescent="0.35">
       <c r="A29" s="3" t="s">
         <v>21</v>
       </c>
@@ -4041,7 +4046,7 @@
       <c r="F29" s="3"/>
       <c r="G29" s="4"/>
     </row>
-    <row r="30" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A30" s="3" t="s">
         <v>25</v>
       </c>
@@ -4058,7 +4063,7 @@
       <c r="F30" s="3"/>
       <c r="G30" s="4"/>
     </row>
-    <row r="31" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A31" s="3" t="s">
         <v>28</v>
       </c>
@@ -4075,7 +4080,7 @@
       <c r="F31" s="3"/>
       <c r="G31" s="4"/>
     </row>
-    <row r="32" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A32" s="3" t="s">
         <v>31</v>
       </c>
@@ -4092,7 +4097,7 @@
       <c r="F32" s="3"/>
       <c r="G32" s="4"/>
     </row>
-    <row r="33" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:7" ht="58" x14ac:dyDescent="0.35">
       <c r="A33" s="3" t="s">
         <v>35</v>
       </c>
@@ -4109,7 +4114,7 @@
       <c r="F33" s="3"/>
       <c r="G33" s="4"/>
     </row>
-    <row r="34" spans="1:7" ht="120" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:7" ht="116" x14ac:dyDescent="0.35">
       <c r="A34" s="3" t="s">
         <v>36</v>
       </c>
@@ -4128,7 +4133,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="35" spans="1:7" ht="120" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:7" ht="116" x14ac:dyDescent="0.35">
       <c r="A35" s="3" t="s">
         <v>37</v>
       </c>
@@ -4147,7 +4152,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="36" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:7" ht="58" x14ac:dyDescent="0.35">
       <c r="A36" s="3" t="s">
         <v>38</v>
       </c>
@@ -4166,7 +4171,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="37" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:7" ht="58" x14ac:dyDescent="0.35">
       <c r="A37" s="3" t="s">
         <v>39</v>
       </c>
@@ -4185,7 +4190,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="38" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:7" ht="58" x14ac:dyDescent="0.35">
       <c r="A38" s="3" t="s">
         <v>162</v>
       </c>
@@ -4204,7 +4209,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="39" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:7" ht="58" x14ac:dyDescent="0.35">
       <c r="A39" s="3" t="s">
         <v>163</v>
       </c>
@@ -4223,7 +4228,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="40" spans="1:7" ht="75" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:7" ht="58" x14ac:dyDescent="0.35">
       <c r="A40" s="3" t="s">
         <v>40</v>
       </c>
@@ -4242,7 +4247,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="41" spans="1:7" ht="75" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:7" ht="58" x14ac:dyDescent="0.35">
       <c r="A41" s="3" t="s">
         <v>41</v>
       </c>
@@ -4261,7 +4266,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="42" spans="1:7" ht="90" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:7" ht="87" x14ac:dyDescent="0.35">
       <c r="A42" s="3" t="s">
         <v>42</v>
       </c>
@@ -4280,7 +4285,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="43" spans="1:7" ht="90" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:7" ht="87" x14ac:dyDescent="0.35">
       <c r="A43" s="3" t="s">
         <v>43</v>
       </c>
@@ -4299,7 +4304,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A44" s="3"/>
       <c r="B44" s="3"/>
       <c r="C44" s="3"/>
@@ -4308,7 +4313,7 @@
       <c r="F44" s="3"/>
       <c r="G44" s="4"/>
     </row>
-    <row r="45" spans="1:7" ht="105" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:7" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A45" s="9" t="s">
         <v>172</v>
       </c>
@@ -4331,7 +4336,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="46" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A46" s="3" t="s">
         <v>10</v>
       </c>
@@ -4348,7 +4353,7 @@
       <c r="F46" s="3"/>
       <c r="G46" s="4"/>
     </row>
-    <row r="47" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A47" s="3" t="s">
         <v>13</v>
       </c>
@@ -4365,7 +4370,7 @@
       <c r="F47" s="3"/>
       <c r="G47" s="4"/>
     </row>
-    <row r="48" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A48" s="3" t="s">
         <v>16</v>
       </c>
@@ -4382,7 +4387,7 @@
       <c r="F48" s="3"/>
       <c r="G48" s="4"/>
     </row>
-    <row r="49" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A49" s="3" t="s">
         <v>20</v>
       </c>
@@ -4399,7 +4404,7 @@
       <c r="F49" s="3"/>
       <c r="G49" s="4"/>
     </row>
-    <row r="50" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A50" s="3" t="s">
         <v>24</v>
       </c>
@@ -4416,7 +4421,7 @@
       <c r="F50" s="3"/>
       <c r="G50" s="4"/>
     </row>
-    <row r="51" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A51" s="3" t="s">
         <v>27</v>
       </c>
@@ -4433,7 +4438,7 @@
       <c r="F51" s="3"/>
       <c r="G51" s="4"/>
     </row>
-    <row r="52" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A52" s="3" t="s">
         <v>30</v>
       </c>
@@ -4450,7 +4455,7 @@
       <c r="F52" s="3"/>
       <c r="G52" s="4"/>
     </row>
-    <row r="53" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A53" s="3" t="s">
         <v>34</v>
       </c>
@@ -4467,7 +4472,7 @@
       <c r="F53" s="3"/>
       <c r="G53" s="4"/>
     </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A54" s="3"/>
       <c r="B54" s="3"/>
       <c r="C54" s="3"/>
@@ -4476,7 +4481,7 @@
       <c r="F54" s="3"/>
       <c r="G54" s="4"/>
     </row>
-    <row r="55" spans="1:7" ht="75" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:7" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A55" s="11" t="s">
         <v>173</v>
       </c>
@@ -4499,7 +4504,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A56" s="3" t="s">
         <v>44</v>
       </c>
@@ -4516,7 +4521,7 @@
       <c r="F56" s="3"/>
       <c r="G56" s="4"/>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A57" s="3" t="s">
         <v>45</v>
       </c>
@@ -4535,7 +4540,7 @@
       </c>
       <c r="G57" s="4"/>
     </row>
-    <row r="58" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A58" s="3" t="s">
         <v>46</v>
       </c>
@@ -4554,7 +4559,7 @@
       </c>
       <c r="G58" s="4"/>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A59" s="3" t="s">
         <v>47</v>
       </c>
@@ -4571,7 +4576,7 @@
       <c r="F59" s="3"/>
       <c r="G59" s="4"/>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A60" s="3" t="s">
         <v>48</v>
       </c>

</xml_diff>

<commit_message>
Added functions for the trade-off plot, including utility functions.
</commit_message>
<xml_diff>
--- a/data-raw/Manuscript_Generic_Example.xlsx
+++ b/data-raw/Manuscript_Generic_Example.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28925"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lgaka\Downloads\brpubVJCE\data-raw\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fengh\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45E440DB-7E6D-4DAC-9237-F4DD7BC63BA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7EF72D8-26E5-477D-81E3-22566F9AF6AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1470" yWindow="735" windowWidth="19793" windowHeight="12765" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Example Effects Table" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="639" uniqueCount="200">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="639" uniqueCount="201">
   <si>
     <t>Factor</t>
   </si>
@@ -651,6 +651,10 @@
   </si>
   <si>
     <t>Risk 3</t>
+  </si>
+  <si>
+    <t>Risk 3</t>
+    <phoneticPr fontId="5" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -658,13 +662,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="0.000"/>
+    <numFmt numFmtId="176" formatCode="0.000"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="等线"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -672,7 +676,7 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="等线"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -680,28 +684,35 @@
       <b/>
       <sz val="12"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="等线"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="12"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="等线"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="12"/>
       <color rgb="FF333333"/>
-      <name val="Calibri"/>
+      <name val="等线"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="8"/>
-      <name val="Calibri"/>
+      <name val="等线"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="等线"/>
+      <family val="3"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -872,7 +883,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="3" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="176" fontId="3" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -889,14 +900,14 @@
     <xf numFmtId="0" fontId="0" fillId="13" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="13" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="176" fontId="0" fillId="13" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="176" fontId="0" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="176" fontId="0" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="176" fontId="0" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="常规" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1175,24 +1186,24 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AY25"/>
-  <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.73046875" defaultRowHeight="13.9" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="2" max="2" width="22.1796875" customWidth="1"/>
-    <col min="3" max="3" width="20.81640625" customWidth="1"/>
-    <col min="4" max="4" width="26.453125" customWidth="1"/>
-    <col min="5" max="5" width="14.7265625" customWidth="1"/>
-    <col min="6" max="6" width="10.54296875" customWidth="1"/>
-    <col min="7" max="7" width="12.26953125" customWidth="1"/>
-    <col min="15" max="15" width="9.1796875" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="11.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.19921875" customWidth="1"/>
+    <col min="3" max="3" width="20.796875" customWidth="1"/>
+    <col min="4" max="4" width="26.46484375" customWidth="1"/>
+    <col min="5" max="5" width="14.73046875" customWidth="1"/>
+    <col min="6" max="6" width="10.53125" customWidth="1"/>
+    <col min="7" max="7" width="12.265625" customWidth="1"/>
+    <col min="15" max="15" width="9.19921875" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="11.796875" bestFit="1" customWidth="1"/>
     <col min="22" max="22" width="12" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="10.26953125" customWidth="1"/>
-    <col min="24" max="24" width="9.1796875" customWidth="1"/>
-    <col min="29" max="29" width="9.1796875" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="11.81640625" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="10.265625" customWidth="1"/>
+    <col min="24" max="24" width="9.19921875" customWidth="1"/>
+    <col min="29" max="29" width="9.19921875" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="11.796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:51" s="23" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:51" s="23" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A1" s="24" t="s">
         <v>0</v>
       </c>
@@ -1347,7 +1358,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="2" spans="1:51" s="23" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:51" s="23" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A2" s="23" t="s">
         <v>49</v>
       </c>
@@ -1423,7 +1434,7 @@
       <c r="AI2" s="33"/>
       <c r="AJ2" s="33"/>
     </row>
-    <row r="3" spans="1:51" s="23" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:51" s="23" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A3" s="23" t="s">
         <v>49</v>
       </c>
@@ -1495,7 +1506,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:51" s="23" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:51" s="23" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A4" s="23" t="s">
         <v>49</v>
       </c>
@@ -1564,7 +1575,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:51" s="23" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:51" s="23" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A5" s="23" t="s">
         <v>61</v>
       </c>
@@ -1656,7 +1667,7 @@
       <c r="AI5" s="33"/>
       <c r="AJ5" s="33"/>
     </row>
-    <row r="6" spans="1:51" s="23" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:51" s="23" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A6" s="23" t="s">
         <v>61</v>
       </c>
@@ -1745,7 +1756,7 @@
       <c r="AI6" s="33"/>
       <c r="AJ6" s="33"/>
     </row>
-    <row r="7" spans="1:51" s="23" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:51" s="23" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A7" s="23" t="s">
         <v>61</v>
       </c>
@@ -1835,7 +1846,7 @@
       <c r="AI7" s="33"/>
       <c r="AJ7" s="33"/>
     </row>
-    <row r="8" spans="1:51" s="30" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:51" s="30" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A8" s="30" t="s">
         <v>49</v>
       </c>
@@ -1911,7 +1922,7 @@
       <c r="AI8" s="33"/>
       <c r="AJ8" s="33"/>
     </row>
-    <row r="9" spans="1:51" s="30" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:51" s="30" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A9" s="30" t="s">
         <v>49</v>
       </c>
@@ -1980,7 +1991,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="10" spans="1:51" s="30" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:51" s="30" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A10" s="30" t="s">
         <v>49</v>
       </c>
@@ -2051,7 +2062,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="11" spans="1:51" s="30" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:51" s="30" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A11" s="30" t="s">
         <v>61</v>
       </c>
@@ -2143,7 +2154,7 @@
       <c r="AI11" s="33"/>
       <c r="AJ11" s="33"/>
     </row>
-    <row r="12" spans="1:51" s="30" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:51" s="30" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A12" s="30" t="s">
         <v>61</v>
       </c>
@@ -2233,7 +2244,7 @@
       <c r="AI12" s="33"/>
       <c r="AJ12" s="33"/>
     </row>
-    <row r="13" spans="1:51" s="30" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:51" s="30" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A13" s="30" t="s">
         <v>61</v>
       </c>
@@ -2241,7 +2252,7 @@
         <v>175</v>
       </c>
       <c r="C13" s="30" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="D13" s="30" t="s">
         <v>178</v>
@@ -2323,7 +2334,7 @@
       <c r="AI13" s="33"/>
       <c r="AJ13" s="33"/>
     </row>
-    <row r="14" spans="1:51" s="31" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:51" s="31" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A14" s="31" t="s">
         <v>49</v>
       </c>
@@ -2399,7 +2410,7 @@
       <c r="AI14" s="33"/>
       <c r="AJ14" s="33"/>
     </row>
-    <row r="15" spans="1:51" s="31" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:51" s="31" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A15" s="31" t="s">
         <v>49</v>
       </c>
@@ -2468,7 +2479,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="16" spans="1:51" s="31" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:51" s="31" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A16" s="31" t="s">
         <v>49</v>
       </c>
@@ -2539,7 +2550,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="17" spans="1:36" s="31" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:36" s="31" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A17" s="31" t="s">
         <v>61</v>
       </c>
@@ -2631,7 +2642,7 @@
       <c r="AI17" s="33"/>
       <c r="AJ17" s="33"/>
     </row>
-    <row r="18" spans="1:36" s="31" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:36" s="31" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A18" s="31" t="s">
         <v>61</v>
       </c>
@@ -2721,7 +2732,7 @@
       <c r="AI18" s="33"/>
       <c r="AJ18" s="33"/>
     </row>
-    <row r="19" spans="1:36" s="31" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:36" s="31" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A19" s="31" t="s">
         <v>61</v>
       </c>
@@ -2811,7 +2822,7 @@
       <c r="AI19" s="33"/>
       <c r="AJ19" s="33"/>
     </row>
-    <row r="20" spans="1:36" s="32" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:36" s="32" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A20" s="32" t="s">
         <v>49</v>
       </c>
@@ -2887,7 +2898,7 @@
       <c r="AI20" s="33"/>
       <c r="AJ20" s="33"/>
     </row>
-    <row r="21" spans="1:36" s="32" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:36" s="32" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A21" s="32" t="s">
         <v>49</v>
       </c>
@@ -2966,7 +2977,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="22" spans="1:36" s="32" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:36" s="32" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A22" s="32" t="s">
         <v>49</v>
       </c>
@@ -3038,7 +3049,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="23" spans="1:36" s="32" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:36" s="32" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A23" s="32" t="s">
         <v>61</v>
       </c>
@@ -3131,7 +3142,7 @@
       <c r="AI23" s="33"/>
       <c r="AJ23" s="33"/>
     </row>
-    <row r="24" spans="1:36" s="32" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:36" s="32" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A24" s="32" t="s">
         <v>61</v>
       </c>
@@ -3221,7 +3232,7 @@
       <c r="AI24" s="33"/>
       <c r="AJ24" s="33"/>
     </row>
-    <row r="25" spans="1:36" s="32" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:36" s="32" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A25" s="32" t="s">
         <v>61</v>
       </c>
@@ -3321,14 +3332,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5D4A282F-FA68-4BC3-9814-08A63A8C35E3}">
   <dimension ref="A1:C16"/>
-  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="16.453125" style="16" customWidth="1"/>
-    <col min="2" max="2" width="7.1796875" style="16" customWidth="1"/>
-    <col min="3" max="3" width="12.26953125" style="17" customWidth="1"/>
+    <col min="1" max="1" width="16.46484375" style="16" customWidth="1"/>
+    <col min="2" max="2" width="7.19921875" style="16" customWidth="1"/>
+    <col min="3" max="3" width="12.265625" style="17" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" s="15" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" s="15" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A1" s="18" t="s">
         <v>179</v>
       </c>
@@ -3339,7 +3350,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" s="20" t="s">
         <v>182</v>
       </c>
@@ -3350,7 +3361,7 @@
         <v>0.02</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" s="20" t="s">
         <v>182</v>
       </c>
@@ -3361,7 +3372,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" s="20" t="s">
         <v>182</v>
       </c>
@@ -3372,7 +3383,7 @@
         <v>0.25</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A5" s="20" t="s">
         <v>181</v>
       </c>
@@ -3383,7 +3394,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A6" s="20" t="s">
         <v>181</v>
       </c>
@@ -3394,7 +3405,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A7" s="20" t="s">
         <v>181</v>
       </c>
@@ -3405,7 +3416,7 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A8" s="20" t="s">
         <v>183</v>
       </c>
@@ -3416,7 +3427,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A9" s="20" t="s">
         <v>183</v>
       </c>
@@ -3427,7 +3438,7 @@
         <v>0.25</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A10" s="20" t="s">
         <v>183</v>
       </c>
@@ -3438,7 +3449,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A11" s="22" t="s">
         <v>184</v>
       </c>
@@ -3449,7 +3460,7 @@
         <v>1E-3</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A12" s="20" t="s">
         <v>184</v>
       </c>
@@ -3460,7 +3471,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A13" s="20" t="s">
         <v>184</v>
       </c>
@@ -3471,7 +3482,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A14" s="20" t="s">
         <v>185</v>
       </c>
@@ -3482,7 +3493,7 @@
         <v>1E-3</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A15" s="20" t="s">
         <v>185</v>
       </c>
@@ -3493,7 +3504,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A16" s="20" t="s">
         <v>185</v>
       </c>
@@ -3505,6 +3516,7 @@
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="6" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -3512,18 +3524,18 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F7B77BDC-7246-43E5-B2E5-9DD908E43155}">
   <dimension ref="A1:G60"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="13.9" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="17.453125" style="13" customWidth="1"/>
-    <col min="2" max="2" width="21.81640625" style="13" customWidth="1"/>
-    <col min="3" max="3" width="42.54296875" style="13" customWidth="1"/>
-    <col min="4" max="4" width="9.7265625" style="14" customWidth="1"/>
+    <col min="1" max="1" width="17.46484375" style="13" customWidth="1"/>
+    <col min="2" max="2" width="21.796875" style="13" customWidth="1"/>
+    <col min="3" max="3" width="42.53125" style="13" customWidth="1"/>
+    <col min="4" max="4" width="9.73046875" style="14" customWidth="1"/>
     <col min="5" max="5" width="18" style="13" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="22.54296875" style="13" customWidth="1"/>
-    <col min="7" max="7" width="35.26953125" style="14" customWidth="1"/>
+    <col min="6" max="6" width="22.53125" style="13" customWidth="1"/>
+    <col min="7" max="7" width="35.265625" style="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" s="1" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" s="1" customFormat="1" ht="97.15" x14ac:dyDescent="0.4">
       <c r="A1" s="2" t="s">
         <v>170</v>
       </c>
@@ -3546,7 +3558,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A2" s="3" t="s">
         <v>0</v>
       </c>
@@ -3565,7 +3577,7 @@
       <c r="F2" s="3"/>
       <c r="G2" s="4"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
@@ -3584,7 +3596,7 @@
       </c>
       <c r="G3" s="4"/>
     </row>
-    <row r="4" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:7" ht="41.65" x14ac:dyDescent="0.4">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -3603,7 +3615,7 @@
       </c>
       <c r="G4" s="4"/>
     </row>
-    <row r="5" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:7" ht="27.75" x14ac:dyDescent="0.4">
       <c r="A5" s="3" t="s">
         <v>3</v>
       </c>
@@ -3622,7 +3634,7 @@
       </c>
       <c r="G5" s="4"/>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A6" s="3" t="s">
         <v>4</v>
       </c>
@@ -3641,7 +3653,7 @@
       <c r="F6" s="3"/>
       <c r="G6" s="4"/>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A7" s="3" t="s">
         <v>6</v>
       </c>
@@ -3660,7 +3672,7 @@
       <c r="F7" s="3"/>
       <c r="G7" s="4"/>
     </row>
-    <row r="8" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:7" ht="27.75" x14ac:dyDescent="0.4">
       <c r="A8" s="3" t="s">
         <v>7</v>
       </c>
@@ -3681,7 +3693,7 @@
       </c>
       <c r="G8" s="4"/>
     </row>
-    <row r="9" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:7" ht="27.75" x14ac:dyDescent="0.4">
       <c r="A9" s="3" t="s">
         <v>8</v>
       </c>
@@ -3702,7 +3714,7 @@
       </c>
       <c r="G9" s="4"/>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A10" s="3" t="s">
         <v>9</v>
       </c>
@@ -3721,7 +3733,7 @@
       </c>
       <c r="G10" s="4"/>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A11" s="3" t="s">
         <v>23</v>
       </c>
@@ -3740,7 +3752,7 @@
       <c r="F11" s="3"/>
       <c r="G11" s="4"/>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A12" s="3" t="s">
         <v>22</v>
       </c>
@@ -3759,7 +3771,7 @@
       <c r="F12" s="3"/>
       <c r="G12" s="4"/>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A13" s="3"/>
       <c r="B13" s="3"/>
       <c r="C13" s="3"/>
@@ -3768,7 +3780,7 @@
       <c r="F13" s="3"/>
       <c r="G13" s="4"/>
     </row>
-    <row r="14" spans="1:7" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:7" ht="97.15" x14ac:dyDescent="0.4">
       <c r="A14" s="5" t="s">
         <v>169</v>
       </c>
@@ -3791,7 +3803,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="15" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:7" ht="27.75" x14ac:dyDescent="0.4">
       <c r="A15" s="3" t="s">
         <v>5</v>
       </c>
@@ -3810,7 +3822,7 @@
       <c r="F15" s="3"/>
       <c r="G15" s="4"/>
     </row>
-    <row r="16" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:7" ht="41.65" x14ac:dyDescent="0.4">
       <c r="A16" s="3" t="s">
         <v>12</v>
       </c>
@@ -3827,7 +3839,7 @@
       <c r="F16" s="3"/>
       <c r="G16" s="4"/>
     </row>
-    <row r="17" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:7" ht="55.5" x14ac:dyDescent="0.4">
       <c r="A17" s="3" t="s">
         <v>15</v>
       </c>
@@ -3844,7 +3856,7 @@
       <c r="F17" s="3"/>
       <c r="G17" s="4"/>
     </row>
-    <row r="18" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:7" ht="55.5" x14ac:dyDescent="0.4">
       <c r="A18" s="3" t="s">
         <v>18</v>
       </c>
@@ -3861,7 +3873,7 @@
       <c r="F18" s="3"/>
       <c r="G18" s="4"/>
     </row>
-    <row r="19" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A19" s="3" t="s">
         <v>19</v>
       </c>
@@ -3878,7 +3890,7 @@
       <c r="F19" s="3"/>
       <c r="G19" s="4"/>
     </row>
-    <row r="20" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:7" ht="41.65" x14ac:dyDescent="0.4">
       <c r="A20" s="3" t="s">
         <v>26</v>
       </c>
@@ -3895,7 +3907,7 @@
       <c r="F20" s="3"/>
       <c r="G20" s="4"/>
     </row>
-    <row r="21" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:7" ht="55.5" x14ac:dyDescent="0.4">
       <c r="A21" s="3" t="s">
         <v>29</v>
       </c>
@@ -3912,7 +3924,7 @@
       <c r="F21" s="3"/>
       <c r="G21" s="4"/>
     </row>
-    <row r="22" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:7" ht="55.5" x14ac:dyDescent="0.4">
       <c r="A22" s="3" t="s">
         <v>32</v>
       </c>
@@ -3929,7 +3941,7 @@
       <c r="F22" s="3"/>
       <c r="G22" s="4"/>
     </row>
-    <row r="23" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:7" ht="27.75" x14ac:dyDescent="0.4">
       <c r="A23" s="3" t="s">
         <v>33</v>
       </c>
@@ -3946,7 +3958,7 @@
       <c r="F23" s="3"/>
       <c r="G23" s="4"/>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A24" s="3"/>
       <c r="B24" s="3"/>
       <c r="C24" s="3"/>
@@ -3955,7 +3967,7 @@
       <c r="F24" s="3"/>
       <c r="G24" s="4"/>
     </row>
-    <row r="25" spans="1:7" ht="87" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:7" ht="83.25" x14ac:dyDescent="0.4">
       <c r="A25" s="7" t="s">
         <v>171</v>
       </c>
@@ -3978,7 +3990,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="26" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:7" ht="27.75" x14ac:dyDescent="0.4">
       <c r="A26" s="3" t="s">
         <v>11</v>
       </c>
@@ -3995,7 +4007,7 @@
       <c r="F26" s="3"/>
       <c r="G26" s="4"/>
     </row>
-    <row r="27" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:7" ht="41.65" x14ac:dyDescent="0.4">
       <c r="A27" s="3" t="s">
         <v>14</v>
       </c>
@@ -4012,7 +4024,7 @@
       <c r="F27" s="3"/>
       <c r="G27" s="4"/>
     </row>
-    <row r="28" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:7" ht="41.65" x14ac:dyDescent="0.4">
       <c r="A28" s="3" t="s">
         <v>17</v>
       </c>
@@ -4029,7 +4041,7 @@
       <c r="F28" s="3"/>
       <c r="G28" s="4"/>
     </row>
-    <row r="29" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:7" ht="55.5" x14ac:dyDescent="0.4">
       <c r="A29" s="3" t="s">
         <v>21</v>
       </c>
@@ -4046,7 +4058,7 @@
       <c r="F29" s="3"/>
       <c r="G29" s="4"/>
     </row>
-    <row r="30" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:7" ht="27.75" x14ac:dyDescent="0.4">
       <c r="A30" s="3" t="s">
         <v>25</v>
       </c>
@@ -4063,7 +4075,7 @@
       <c r="F30" s="3"/>
       <c r="G30" s="4"/>
     </row>
-    <row r="31" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:7" ht="41.65" x14ac:dyDescent="0.4">
       <c r="A31" s="3" t="s">
         <v>28</v>
       </c>
@@ -4080,7 +4092,7 @@
       <c r="F31" s="3"/>
       <c r="G31" s="4"/>
     </row>
-    <row r="32" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:7" ht="41.65" x14ac:dyDescent="0.4">
       <c r="A32" s="3" t="s">
         <v>31</v>
       </c>
@@ -4097,7 +4109,7 @@
       <c r="F32" s="3"/>
       <c r="G32" s="4"/>
     </row>
-    <row r="33" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:7" ht="55.5" x14ac:dyDescent="0.4">
       <c r="A33" s="3" t="s">
         <v>35</v>
       </c>
@@ -4114,7 +4126,7 @@
       <c r="F33" s="3"/>
       <c r="G33" s="4"/>
     </row>
-    <row r="34" spans="1:7" ht="116" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:7" ht="111" x14ac:dyDescent="0.4">
       <c r="A34" s="3" t="s">
         <v>36</v>
       </c>
@@ -4133,7 +4145,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="35" spans="1:7" ht="116" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:7" ht="111" x14ac:dyDescent="0.4">
       <c r="A35" s="3" t="s">
         <v>37</v>
       </c>
@@ -4152,7 +4164,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="36" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:7" ht="55.5" x14ac:dyDescent="0.4">
       <c r="A36" s="3" t="s">
         <v>38</v>
       </c>
@@ -4171,7 +4183,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="37" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:7" ht="55.5" x14ac:dyDescent="0.4">
       <c r="A37" s="3" t="s">
         <v>39</v>
       </c>
@@ -4190,7 +4202,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="38" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:7" ht="55.5" x14ac:dyDescent="0.4">
       <c r="A38" s="3" t="s">
         <v>162</v>
       </c>
@@ -4209,7 +4221,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="39" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:7" ht="55.5" x14ac:dyDescent="0.4">
       <c r="A39" s="3" t="s">
         <v>163</v>
       </c>
@@ -4228,7 +4240,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="40" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:7" ht="55.5" x14ac:dyDescent="0.4">
       <c r="A40" s="3" t="s">
         <v>40</v>
       </c>
@@ -4247,7 +4259,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="41" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:7" ht="55.5" x14ac:dyDescent="0.4">
       <c r="A41" s="3" t="s">
         <v>41</v>
       </c>
@@ -4266,7 +4278,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="42" spans="1:7" ht="87" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:7" ht="83.25" x14ac:dyDescent="0.4">
       <c r="A42" s="3" t="s">
         <v>42</v>
       </c>
@@ -4285,7 +4297,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="43" spans="1:7" ht="87" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:7" ht="83.25" x14ac:dyDescent="0.4">
       <c r="A43" s="3" t="s">
         <v>43</v>
       </c>
@@ -4304,7 +4316,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A44" s="3"/>
       <c r="B44" s="3"/>
       <c r="C44" s="3"/>
@@ -4313,7 +4325,7 @@
       <c r="F44" s="3"/>
       <c r="G44" s="4"/>
     </row>
-    <row r="45" spans="1:7" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:7" ht="83.25" x14ac:dyDescent="0.4">
       <c r="A45" s="9" t="s">
         <v>172</v>
       </c>
@@ -4336,7 +4348,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="46" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:7" ht="41.65" x14ac:dyDescent="0.4">
       <c r="A46" s="3" t="s">
         <v>10</v>
       </c>
@@ -4353,7 +4365,7 @@
       <c r="F46" s="3"/>
       <c r="G46" s="4"/>
     </row>
-    <row r="47" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:7" ht="27.75" x14ac:dyDescent="0.4">
       <c r="A47" s="3" t="s">
         <v>13</v>
       </c>
@@ -4370,7 +4382,7 @@
       <c r="F47" s="3"/>
       <c r="G47" s="4"/>
     </row>
-    <row r="48" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:7" ht="27.75" x14ac:dyDescent="0.4">
       <c r="A48" s="3" t="s">
         <v>16</v>
       </c>
@@ -4387,7 +4399,7 @@
       <c r="F48" s="3"/>
       <c r="G48" s="4"/>
     </row>
-    <row r="49" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:7" ht="27.75" x14ac:dyDescent="0.4">
       <c r="A49" s="3" t="s">
         <v>20</v>
       </c>
@@ -4404,7 +4416,7 @@
       <c r="F49" s="3"/>
       <c r="G49" s="4"/>
     </row>
-    <row r="50" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:7" ht="41.65" x14ac:dyDescent="0.4">
       <c r="A50" s="3" t="s">
         <v>24</v>
       </c>
@@ -4421,7 +4433,7 @@
       <c r="F50" s="3"/>
       <c r="G50" s="4"/>
     </row>
-    <row r="51" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:7" ht="27.75" x14ac:dyDescent="0.4">
       <c r="A51" s="3" t="s">
         <v>27</v>
       </c>
@@ -4438,7 +4450,7 @@
       <c r="F51" s="3"/>
       <c r="G51" s="4"/>
     </row>
-    <row r="52" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:7" ht="27.75" x14ac:dyDescent="0.4">
       <c r="A52" s="3" t="s">
         <v>30</v>
       </c>
@@ -4455,7 +4467,7 @@
       <c r="F52" s="3"/>
       <c r="G52" s="4"/>
     </row>
-    <row r="53" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:7" ht="27.75" x14ac:dyDescent="0.4">
       <c r="A53" s="3" t="s">
         <v>34</v>
       </c>
@@ -4472,7 +4484,7 @@
       <c r="F53" s="3"/>
       <c r="G53" s="4"/>
     </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A54" s="3"/>
       <c r="B54" s="3"/>
       <c r="C54" s="3"/>
@@ -4481,7 +4493,7 @@
       <c r="F54" s="3"/>
       <c r="G54" s="4"/>
     </row>
-    <row r="55" spans="1:7" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:7" ht="69.400000000000006" x14ac:dyDescent="0.4">
       <c r="A55" s="11" t="s">
         <v>173</v>
       </c>
@@ -4504,7 +4516,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A56" s="3" t="s">
         <v>44</v>
       </c>
@@ -4521,7 +4533,7 @@
       <c r="F56" s="3"/>
       <c r="G56" s="4"/>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A57" s="3" t="s">
         <v>45</v>
       </c>
@@ -4540,7 +4552,7 @@
       </c>
       <c r="G57" s="4"/>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A58" s="3" t="s">
         <v>46</v>
       </c>
@@ -4559,7 +4571,7 @@
       </c>
       <c r="G58" s="4"/>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A59" s="3" t="s">
         <v>47</v>
       </c>
@@ -4576,7 +4588,7 @@
       <c r="F59" s="3"/>
       <c r="G59" s="4"/>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A60" s="3" t="s">
         <v>48</v>
       </c>
@@ -4594,11 +4606,32 @@
       <c r="G60" s="4"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="6" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="e522a4ea-6824-496f-8ffe-e074cc291ac0">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="8080ce30-d5ea-40e8-a48f-b77958a33e4e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100CBEA71EDBDE86541B7589EDD610CDCA6" ma:contentTypeVersion="10" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="6135c02e9fba22fa14c95532ff73e585">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="e522a4ea-6824-496f-8ffe-e074cc291ac0" xmlns:ns3="8080ce30-d5ea-40e8-a48f-b77958a33e4e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4c9beda59bcc2e0dae0951e4601e1985" ns2:_="" ns3:_="">
     <xsd:import namespace="e522a4ea-6824-496f-8ffe-e074cc291ac0"/>
@@ -4789,27 +4822,32 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{13FE4927-61BE-41A1-B367-1B1C5D848E2B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="e522a4ea-6824-496f-8ffe-e074cc291ac0"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="8080ce30-d5ea-40e8-a48f-b77958a33e4e"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="e522a4ea-6824-496f-8ffe-e074cc291ac0">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="8080ce30-d5ea-40e8-a48f-b77958a33e4e" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8E8BB74B-0686-4136-81AA-6AA3532E32A8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EF3A5692-B908-4374-9724-9509DDA5EAF8}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -4826,29 +4864,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8E8BB74B-0686-4136-81AA-6AA3532E32A8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{13FE4927-61BE-41A1-B367-1B1C5D848E2B}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="e522a4ea-6824-496f-8ffe-e074cc291ac0"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="8080ce30-d5ea-40e8-a48f-b77958a33e4e"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
feat: implement axis reversal for benefit outcomes with negative thresholds
- Add axis reversal logic for benefit outcomes when direction='less' or threshold < 0
- Reverse x-axis scale and coordinate system while maintaining consistent favours labels
- Enhance shaded region logic with proper reversed axis handling
- Fix prepare_forest_dot_data to handle missing binary columns (Prop1/Prop2)
- Add conditional processing to avoid evaluating non-existent columns
- Update documentation with axis reversal examples and clinical use cases
- Add comprehensive test coverage for axis reversal functionality
- Clean up README.Rmd with proper code examples and realistic thresholds

Breaking changes: None - fully backwards compatible
Tests: All 11 tests passing including new axis reversal test

Resolves: Enhancement for negative treatment difference visualization in benefit outcomes
</commit_message>
<xml_diff>
--- a/data-raw/Manuscript_Generic_Example.xlsx
+++ b/data-raw/Manuscript_Generic_Example.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10913"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lgaka\Downloads\brpubVJCE\data-raw\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lvgk/Downloads/brpubVJCE/data-raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45E440DB-7E6D-4DAC-9237-F4DD7BC63BA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E049493-3C93-E54B-A2E9-2608BD3C84A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="30240" windowHeight="17900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Example Effects Table" sheetId="1" r:id="rId1"/>
@@ -1175,24 +1175,24 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AY25"/>
-  <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="22.1796875" customWidth="1"/>
-    <col min="3" max="3" width="20.81640625" customWidth="1"/>
-    <col min="4" max="4" width="26.453125" customWidth="1"/>
-    <col min="5" max="5" width="14.7265625" customWidth="1"/>
-    <col min="6" max="6" width="10.54296875" customWidth="1"/>
-    <col min="7" max="7" width="12.26953125" customWidth="1"/>
-    <col min="15" max="15" width="9.1796875" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="11.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.1640625" customWidth="1"/>
+    <col min="3" max="3" width="20.83203125" customWidth="1"/>
+    <col min="4" max="4" width="26.5" customWidth="1"/>
+    <col min="5" max="5" width="14.6640625" customWidth="1"/>
+    <col min="6" max="6" width="10.5" customWidth="1"/>
+    <col min="7" max="7" width="12.33203125" customWidth="1"/>
+    <col min="15" max="15" width="9.1640625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="11.83203125" bestFit="1" customWidth="1"/>
     <col min="22" max="22" width="12" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="10.26953125" customWidth="1"/>
-    <col min="24" max="24" width="9.1796875" customWidth="1"/>
-    <col min="29" max="29" width="9.1796875" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="11.81640625" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="10.33203125" customWidth="1"/>
+    <col min="24" max="24" width="9.1640625" customWidth="1"/>
+    <col min="29" max="29" width="9.1640625" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="11.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:51" s="23" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:51" s="23" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="24" t="s">
         <v>0</v>
       </c>
@@ -1347,7 +1347,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="2" spans="1:51" s="23" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:51" s="23" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A2" s="23" t="s">
         <v>49</v>
       </c>
@@ -1423,7 +1423,7 @@
       <c r="AI2" s="33"/>
       <c r="AJ2" s="33"/>
     </row>
-    <row r="3" spans="1:51" s="23" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:51" s="23" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A3" s="23" t="s">
         <v>49</v>
       </c>
@@ -1467,11 +1467,11 @@
       <c r="R3" s="33"/>
       <c r="S3" s="33"/>
       <c r="T3" s="34">
-        <v>65</v>
+        <v>20</v>
       </c>
       <c r="U3" s="34"/>
       <c r="V3" s="34">
-        <v>63</v>
+        <v>16</v>
       </c>
       <c r="W3" s="23" t="s">
         <v>55</v>
@@ -1488,14 +1488,14 @@
       <c r="AF3" s="33"/>
       <c r="AG3" s="33"/>
       <c r="AH3" s="34">
-        <v>20</v>
+        <v>65</v>
       </c>
       <c r="AI3" s="34"/>
       <c r="AJ3" s="34">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="4" spans="1:51" s="23" customFormat="1" x14ac:dyDescent="0.35">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="4" spans="1:51" s="23" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A4" s="23" t="s">
         <v>49</v>
       </c>
@@ -1564,7 +1564,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:51" s="23" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:51" s="23" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A5" s="23" t="s">
         <v>61</v>
       </c>
@@ -1656,7 +1656,7 @@
       <c r="AI5" s="33"/>
       <c r="AJ5" s="33"/>
     </row>
-    <row r="6" spans="1:51" s="23" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:51" s="23" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A6" s="23" t="s">
         <v>61</v>
       </c>
@@ -1745,7 +1745,7 @@
       <c r="AI6" s="33"/>
       <c r="AJ6" s="33"/>
     </row>
-    <row r="7" spans="1:51" s="23" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:51" s="23" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A7" s="23" t="s">
         <v>61</v>
       </c>
@@ -1835,7 +1835,7 @@
       <c r="AI7" s="33"/>
       <c r="AJ7" s="33"/>
     </row>
-    <row r="8" spans="1:51" s="30" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:51" s="30" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A8" s="30" t="s">
         <v>49</v>
       </c>
@@ -1911,7 +1911,7 @@
       <c r="AI8" s="33"/>
       <c r="AJ8" s="33"/>
     </row>
-    <row r="9" spans="1:51" s="30" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:51" s="30" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A9" s="30" t="s">
         <v>49</v>
       </c>
@@ -1980,7 +1980,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="10" spans="1:51" s="30" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:51" s="30" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A10" s="30" t="s">
         <v>49</v>
       </c>
@@ -2051,7 +2051,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="11" spans="1:51" s="30" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:51" s="30" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A11" s="30" t="s">
         <v>61</v>
       </c>
@@ -2143,7 +2143,7 @@
       <c r="AI11" s="33"/>
       <c r="AJ11" s="33"/>
     </row>
-    <row r="12" spans="1:51" s="30" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:51" s="30" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A12" s="30" t="s">
         <v>61</v>
       </c>
@@ -2233,7 +2233,7 @@
       <c r="AI12" s="33"/>
       <c r="AJ12" s="33"/>
     </row>
-    <row r="13" spans="1:51" s="30" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:51" s="30" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A13" s="30" t="s">
         <v>61</v>
       </c>
@@ -2323,7 +2323,7 @@
       <c r="AI13" s="33"/>
       <c r="AJ13" s="33"/>
     </row>
-    <row r="14" spans="1:51" s="31" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:51" s="31" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A14" s="31" t="s">
         <v>49</v>
       </c>
@@ -2399,7 +2399,7 @@
       <c r="AI14" s="33"/>
       <c r="AJ14" s="33"/>
     </row>
-    <row r="15" spans="1:51" s="31" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:51" s="31" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A15" s="31" t="s">
         <v>49</v>
       </c>
@@ -2468,7 +2468,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="16" spans="1:51" s="31" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:51" s="31" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A16" s="31" t="s">
         <v>49</v>
       </c>
@@ -2539,7 +2539,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="17" spans="1:36" s="31" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:36" s="31" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A17" s="31" t="s">
         <v>61</v>
       </c>
@@ -2631,7 +2631,7 @@
       <c r="AI17" s="33"/>
       <c r="AJ17" s="33"/>
     </row>
-    <row r="18" spans="1:36" s="31" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:36" s="31" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A18" s="31" t="s">
         <v>61</v>
       </c>
@@ -2721,7 +2721,7 @@
       <c r="AI18" s="33"/>
       <c r="AJ18" s="33"/>
     </row>
-    <row r="19" spans="1:36" s="31" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:36" s="31" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A19" s="31" t="s">
         <v>61</v>
       </c>
@@ -2811,7 +2811,7 @@
       <c r="AI19" s="33"/>
       <c r="AJ19" s="33"/>
     </row>
-    <row r="20" spans="1:36" s="32" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:36" s="32" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A20" s="32" t="s">
         <v>49</v>
       </c>
@@ -2887,7 +2887,7 @@
       <c r="AI20" s="33"/>
       <c r="AJ20" s="33"/>
     </row>
-    <row r="21" spans="1:36" s="32" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:36" s="32" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A21" s="32" t="s">
         <v>49</v>
       </c>
@@ -2966,7 +2966,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="22" spans="1:36" s="32" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:36" s="32" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A22" s="32" t="s">
         <v>49</v>
       </c>
@@ -3038,7 +3038,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="23" spans="1:36" s="32" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:36" s="32" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A23" s="32" t="s">
         <v>61</v>
       </c>
@@ -3131,7 +3131,7 @@
       <c r="AI23" s="33"/>
       <c r="AJ23" s="33"/>
     </row>
-    <row r="24" spans="1:36" s="32" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:36" s="32" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A24" s="32" t="s">
         <v>61</v>
       </c>
@@ -3221,7 +3221,7 @@
       <c r="AI24" s="33"/>
       <c r="AJ24" s="33"/>
     </row>
-    <row r="25" spans="1:36" s="32" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:36" s="32" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A25" s="32" t="s">
         <v>61</v>
       </c>
@@ -3321,14 +3321,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5D4A282F-FA68-4BC3-9814-08A63A8C35E3}">
   <dimension ref="A1:C16"/>
-  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="16.453125" style="16" customWidth="1"/>
-    <col min="2" max="2" width="7.1796875" style="16" customWidth="1"/>
-    <col min="3" max="3" width="12.26953125" style="17" customWidth="1"/>
+    <col min="1" max="1" width="16.5" style="16" customWidth="1"/>
+    <col min="2" max="2" width="7.1640625" style="16" customWidth="1"/>
+    <col min="3" max="3" width="12.33203125" style="17" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" s="15" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" s="15" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="18" t="s">
         <v>179</v>
       </c>
@@ -3339,7 +3339,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" s="20" t="s">
         <v>182</v>
       </c>
@@ -3350,7 +3350,7 @@
         <v>0.02</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" s="20" t="s">
         <v>182</v>
       </c>
@@ -3361,7 +3361,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" s="20" t="s">
         <v>182</v>
       </c>
@@ -3372,7 +3372,7 @@
         <v>0.25</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" s="20" t="s">
         <v>181</v>
       </c>
@@ -3383,7 +3383,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" s="20" t="s">
         <v>181</v>
       </c>
@@ -3394,7 +3394,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" s="20" t="s">
         <v>181</v>
       </c>
@@ -3405,7 +3405,7 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" s="20" t="s">
         <v>183</v>
       </c>
@@ -3416,7 +3416,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A9" s="20" t="s">
         <v>183</v>
       </c>
@@ -3427,7 +3427,7 @@
         <v>0.25</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A10" s="20" t="s">
         <v>183</v>
       </c>
@@ -3438,7 +3438,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A11" s="22" t="s">
         <v>184</v>
       </c>
@@ -3449,7 +3449,7 @@
         <v>1E-3</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A12" s="20" t="s">
         <v>184</v>
       </c>
@@ -3460,7 +3460,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A13" s="20" t="s">
         <v>184</v>
       </c>
@@ -3471,7 +3471,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A14" s="20" t="s">
         <v>185</v>
       </c>
@@ -3482,7 +3482,7 @@
         <v>1E-3</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A15" s="20" t="s">
         <v>185</v>
       </c>
@@ -3493,7 +3493,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A16" s="20" t="s">
         <v>185</v>
       </c>
@@ -3512,18 +3512,18 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F7B77BDC-7246-43E5-B2E5-9DD908E43155}">
   <dimension ref="A1:G60"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="17.453125" style="13" customWidth="1"/>
-    <col min="2" max="2" width="21.81640625" style="13" customWidth="1"/>
-    <col min="3" max="3" width="42.54296875" style="13" customWidth="1"/>
-    <col min="4" max="4" width="9.7265625" style="14" customWidth="1"/>
+    <col min="1" max="1" width="17.5" style="13" customWidth="1"/>
+    <col min="2" max="2" width="21.83203125" style="13" customWidth="1"/>
+    <col min="3" max="3" width="42.5" style="13" customWidth="1"/>
+    <col min="4" max="4" width="9.6640625" style="14" customWidth="1"/>
     <col min="5" max="5" width="18" style="13" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="22.54296875" style="13" customWidth="1"/>
-    <col min="7" max="7" width="35.26953125" style="14" customWidth="1"/>
+    <col min="6" max="6" width="22.5" style="13" customWidth="1"/>
+    <col min="7" max="7" width="35.33203125" style="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" s="1" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" s="1" customFormat="1" ht="96" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>170</v>
       </c>
@@ -3546,7 +3546,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A2" s="3" t="s">
         <v>0</v>
       </c>
@@ -3565,7 +3565,7 @@
       <c r="F2" s="3"/>
       <c r="G2" s="4"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
@@ -3584,7 +3584,7 @@
       </c>
       <c r="G3" s="4"/>
     </row>
-    <row r="4" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:7" ht="48" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -3603,7 +3603,7 @@
       </c>
       <c r="G4" s="4"/>
     </row>
-    <row r="5" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:7" ht="32" x14ac:dyDescent="0.2">
       <c r="A5" s="3" t="s">
         <v>3</v>
       </c>
@@ -3622,7 +3622,7 @@
       </c>
       <c r="G5" s="4"/>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A6" s="3" t="s">
         <v>4</v>
       </c>
@@ -3641,7 +3641,7 @@
       <c r="F6" s="3"/>
       <c r="G6" s="4"/>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A7" s="3" t="s">
         <v>6</v>
       </c>
@@ -3660,7 +3660,7 @@
       <c r="F7" s="3"/>
       <c r="G7" s="4"/>
     </row>
-    <row r="8" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:7" ht="32" x14ac:dyDescent="0.2">
       <c r="A8" s="3" t="s">
         <v>7</v>
       </c>
@@ -3681,7 +3681,7 @@
       </c>
       <c r="G8" s="4"/>
     </row>
-    <row r="9" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:7" ht="32" x14ac:dyDescent="0.2">
       <c r="A9" s="3" t="s">
         <v>8</v>
       </c>
@@ -3702,7 +3702,7 @@
       </c>
       <c r="G9" s="4"/>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A10" s="3" t="s">
         <v>9</v>
       </c>
@@ -3721,7 +3721,7 @@
       </c>
       <c r="G10" s="4"/>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A11" s="3" t="s">
         <v>23</v>
       </c>
@@ -3740,7 +3740,7 @@
       <c r="F11" s="3"/>
       <c r="G11" s="4"/>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A12" s="3" t="s">
         <v>22</v>
       </c>
@@ -3759,7 +3759,7 @@
       <c r="F12" s="3"/>
       <c r="G12" s="4"/>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" s="3"/>
       <c r="B13" s="3"/>
       <c r="C13" s="3"/>
@@ -3768,7 +3768,7 @@
       <c r="F13" s="3"/>
       <c r="G13" s="4"/>
     </row>
-    <row r="14" spans="1:7" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:7" ht="96" x14ac:dyDescent="0.2">
       <c r="A14" s="5" t="s">
         <v>169</v>
       </c>
@@ -3791,7 +3791,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="15" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:7" ht="32" x14ac:dyDescent="0.2">
       <c r="A15" s="3" t="s">
         <v>5</v>
       </c>
@@ -3810,7 +3810,7 @@
       <c r="F15" s="3"/>
       <c r="G15" s="4"/>
     </row>
-    <row r="16" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:7" ht="48" x14ac:dyDescent="0.2">
       <c r="A16" s="3" t="s">
         <v>12</v>
       </c>
@@ -3827,7 +3827,7 @@
       <c r="F16" s="3"/>
       <c r="G16" s="4"/>
     </row>
-    <row r="17" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:7" ht="64" x14ac:dyDescent="0.2">
       <c r="A17" s="3" t="s">
         <v>15</v>
       </c>
@@ -3844,7 +3844,7 @@
       <c r="F17" s="3"/>
       <c r="G17" s="4"/>
     </row>
-    <row r="18" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:7" ht="64" x14ac:dyDescent="0.2">
       <c r="A18" s="3" t="s">
         <v>18</v>
       </c>
@@ -3861,7 +3861,7 @@
       <c r="F18" s="3"/>
       <c r="G18" s="4"/>
     </row>
-    <row r="19" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A19" s="3" t="s">
         <v>19</v>
       </c>
@@ -3878,7 +3878,7 @@
       <c r="F19" s="3"/>
       <c r="G19" s="4"/>
     </row>
-    <row r="20" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:7" ht="48" x14ac:dyDescent="0.2">
       <c r="A20" s="3" t="s">
         <v>26</v>
       </c>
@@ -3895,7 +3895,7 @@
       <c r="F20" s="3"/>
       <c r="G20" s="4"/>
     </row>
-    <row r="21" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:7" ht="64" x14ac:dyDescent="0.2">
       <c r="A21" s="3" t="s">
         <v>29</v>
       </c>
@@ -3912,7 +3912,7 @@
       <c r="F21" s="3"/>
       <c r="G21" s="4"/>
     </row>
-    <row r="22" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:7" ht="64" x14ac:dyDescent="0.2">
       <c r="A22" s="3" t="s">
         <v>32</v>
       </c>
@@ -3929,7 +3929,7 @@
       <c r="F22" s="3"/>
       <c r="G22" s="4"/>
     </row>
-    <row r="23" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:7" ht="32" x14ac:dyDescent="0.2">
       <c r="A23" s="3" t="s">
         <v>33</v>
       </c>
@@ -3946,7 +3946,7 @@
       <c r="F23" s="3"/>
       <c r="G23" s="4"/>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A24" s="3"/>
       <c r="B24" s="3"/>
       <c r="C24" s="3"/>
@@ -3955,7 +3955,7 @@
       <c r="F24" s="3"/>
       <c r="G24" s="4"/>
     </row>
-    <row r="25" spans="1:7" ht="87" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:7" ht="80" x14ac:dyDescent="0.2">
       <c r="A25" s="7" t="s">
         <v>171</v>
       </c>
@@ -3978,7 +3978,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="26" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:7" ht="32" x14ac:dyDescent="0.2">
       <c r="A26" s="3" t="s">
         <v>11</v>
       </c>
@@ -3995,7 +3995,7 @@
       <c r="F26" s="3"/>
       <c r="G26" s="4"/>
     </row>
-    <row r="27" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:7" ht="48" x14ac:dyDescent="0.2">
       <c r="A27" s="3" t="s">
         <v>14</v>
       </c>
@@ -4012,7 +4012,7 @@
       <c r="F27" s="3"/>
       <c r="G27" s="4"/>
     </row>
-    <row r="28" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:7" ht="48" x14ac:dyDescent="0.2">
       <c r="A28" s="3" t="s">
         <v>17</v>
       </c>
@@ -4029,7 +4029,7 @@
       <c r="F28" s="3"/>
       <c r="G28" s="4"/>
     </row>
-    <row r="29" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:7" ht="64" x14ac:dyDescent="0.2">
       <c r="A29" s="3" t="s">
         <v>21</v>
       </c>
@@ -4046,7 +4046,7 @@
       <c r="F29" s="3"/>
       <c r="G29" s="4"/>
     </row>
-    <row r="30" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:7" ht="32" x14ac:dyDescent="0.2">
       <c r="A30" s="3" t="s">
         <v>25</v>
       </c>
@@ -4063,7 +4063,7 @@
       <c r="F30" s="3"/>
       <c r="G30" s="4"/>
     </row>
-    <row r="31" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:7" ht="48" x14ac:dyDescent="0.2">
       <c r="A31" s="3" t="s">
         <v>28</v>
       </c>
@@ -4080,7 +4080,7 @@
       <c r="F31" s="3"/>
       <c r="G31" s="4"/>
     </row>
-    <row r="32" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:7" ht="48" x14ac:dyDescent="0.2">
       <c r="A32" s="3" t="s">
         <v>31</v>
       </c>
@@ -4097,7 +4097,7 @@
       <c r="F32" s="3"/>
       <c r="G32" s="4"/>
     </row>
-    <row r="33" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:7" ht="64" x14ac:dyDescent="0.2">
       <c r="A33" s="3" t="s">
         <v>35</v>
       </c>
@@ -4114,7 +4114,7 @@
       <c r="F33" s="3"/>
       <c r="G33" s="4"/>
     </row>
-    <row r="34" spans="1:7" ht="116" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:7" ht="128" x14ac:dyDescent="0.2">
       <c r="A34" s="3" t="s">
         <v>36</v>
       </c>
@@ -4133,7 +4133,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="35" spans="1:7" ht="116" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:7" ht="128" x14ac:dyDescent="0.2">
       <c r="A35" s="3" t="s">
         <v>37</v>
       </c>
@@ -4152,7 +4152,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="36" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:7" ht="48" x14ac:dyDescent="0.2">
       <c r="A36" s="3" t="s">
         <v>38</v>
       </c>
@@ -4171,7 +4171,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="37" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:7" ht="48" x14ac:dyDescent="0.2">
       <c r="A37" s="3" t="s">
         <v>39</v>
       </c>
@@ -4190,7 +4190,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="38" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:7" ht="48" x14ac:dyDescent="0.2">
       <c r="A38" s="3" t="s">
         <v>162</v>
       </c>
@@ -4209,7 +4209,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="39" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:7" ht="48" x14ac:dyDescent="0.2">
       <c r="A39" s="3" t="s">
         <v>163</v>
       </c>
@@ -4228,7 +4228,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="40" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:7" ht="64" x14ac:dyDescent="0.2">
       <c r="A40" s="3" t="s">
         <v>40</v>
       </c>
@@ -4247,7 +4247,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="41" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:7" ht="64" x14ac:dyDescent="0.2">
       <c r="A41" s="3" t="s">
         <v>41</v>
       </c>
@@ -4266,7 +4266,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="42" spans="1:7" ht="87" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:7" ht="80" x14ac:dyDescent="0.2">
       <c r="A42" s="3" t="s">
         <v>42</v>
       </c>
@@ -4285,7 +4285,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="43" spans="1:7" ht="87" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:7" ht="80" x14ac:dyDescent="0.2">
       <c r="A43" s="3" t="s">
         <v>43</v>
       </c>
@@ -4304,7 +4304,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A44" s="3"/>
       <c r="B44" s="3"/>
       <c r="C44" s="3"/>
@@ -4313,7 +4313,7 @@
       <c r="F44" s="3"/>
       <c r="G44" s="4"/>
     </row>
-    <row r="45" spans="1:7" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:7" ht="96" x14ac:dyDescent="0.2">
       <c r="A45" s="9" t="s">
         <v>172</v>
       </c>
@@ -4336,7 +4336,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="46" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:7" ht="32" x14ac:dyDescent="0.2">
       <c r="A46" s="3" t="s">
         <v>10</v>
       </c>
@@ -4353,7 +4353,7 @@
       <c r="F46" s="3"/>
       <c r="G46" s="4"/>
     </row>
-    <row r="47" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:7" ht="32" x14ac:dyDescent="0.2">
       <c r="A47" s="3" t="s">
         <v>13</v>
       </c>
@@ -4370,7 +4370,7 @@
       <c r="F47" s="3"/>
       <c r="G47" s="4"/>
     </row>
-    <row r="48" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:7" ht="32" x14ac:dyDescent="0.2">
       <c r="A48" s="3" t="s">
         <v>16</v>
       </c>
@@ -4387,7 +4387,7 @@
       <c r="F48" s="3"/>
       <c r="G48" s="4"/>
     </row>
-    <row r="49" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:7" ht="32" x14ac:dyDescent="0.2">
       <c r="A49" s="3" t="s">
         <v>20</v>
       </c>
@@ -4404,7 +4404,7 @@
       <c r="F49" s="3"/>
       <c r="G49" s="4"/>
     </row>
-    <row r="50" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:7" ht="48" x14ac:dyDescent="0.2">
       <c r="A50" s="3" t="s">
         <v>24</v>
       </c>
@@ -4421,7 +4421,7 @@
       <c r="F50" s="3"/>
       <c r="G50" s="4"/>
     </row>
-    <row r="51" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:7" ht="32" x14ac:dyDescent="0.2">
       <c r="A51" s="3" t="s">
         <v>27</v>
       </c>
@@ -4438,7 +4438,7 @@
       <c r="F51" s="3"/>
       <c r="G51" s="4"/>
     </row>
-    <row r="52" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:7" ht="32" x14ac:dyDescent="0.2">
       <c r="A52" s="3" t="s">
         <v>30</v>
       </c>
@@ -4455,7 +4455,7 @@
       <c r="F52" s="3"/>
       <c r="G52" s="4"/>
     </row>
-    <row r="53" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:7" ht="32" x14ac:dyDescent="0.2">
       <c r="A53" s="3" t="s">
         <v>34</v>
       </c>
@@ -4472,7 +4472,7 @@
       <c r="F53" s="3"/>
       <c r="G53" s="4"/>
     </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A54" s="3"/>
       <c r="B54" s="3"/>
       <c r="C54" s="3"/>
@@ -4481,7 +4481,7 @@
       <c r="F54" s="3"/>
       <c r="G54" s="4"/>
     </row>
-    <row r="55" spans="1:7" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:7" ht="64" x14ac:dyDescent="0.2">
       <c r="A55" s="11" t="s">
         <v>173</v>
       </c>
@@ -4504,7 +4504,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A56" s="3" t="s">
         <v>44</v>
       </c>
@@ -4521,7 +4521,7 @@
       <c r="F56" s="3"/>
       <c r="G56" s="4"/>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A57" s="3" t="s">
         <v>45</v>
       </c>
@@ -4540,7 +4540,7 @@
       </c>
       <c r="G57" s="4"/>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A58" s="3" t="s">
         <v>46</v>
       </c>
@@ -4559,7 +4559,7 @@
       </c>
       <c r="G58" s="4"/>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A59" s="3" t="s">
         <v>47</v>
       </c>
@@ -4576,7 +4576,7 @@
       <c r="F59" s="3"/>
       <c r="G59" s="4"/>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A60" s="3" t="s">
         <v>48</v>
       </c>
@@ -4790,15 +4790,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="e522a4ea-6824-496f-8ffe-e074cc291ac0">
@@ -4807,6 +4798,15 @@
     <TaxCatchAll xmlns="8080ce30-d5ea-40e8-a48f-b77958a33e4e" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4829,14 +4829,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8E8BB74B-0686-4136-81AA-6AA3532E32A8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{13FE4927-61BE-41A1-B367-1B1C5D848E2B}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
@@ -4851,4 +4843,18 @@
     <ds:schemaRef ds:uri="8080ce30-d5ea-40e8-a48f-b77958a33e4e"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8E8BB74B-0686-4136-81AA-6AA3532E32A8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{f743b317-4758-44cb-8b65-8b43e4619766}" enabled="1" method="Standard" siteId="{fdfed7bd-9f6a-44a1-b694-6e39c468c150}" contentBits="0" removed="0"/>
+</clbl:labelList>
 </file>
</xml_diff>

<commit_message>
Checkpoint from VS Code for coding agent session
</commit_message>
<xml_diff>
--- a/data-raw/Manuscript_Generic_Example.xlsx
+++ b/data-raw/Manuscript_Generic_Example.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10913"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fengh\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lvgk/Downloads/brpubVJCE/data-raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7EF72D8-26E5-477D-81E3-22566F9AF6AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E049493-3C93-E54B-A2E9-2608BD3C84A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1470" yWindow="735" windowWidth="19793" windowHeight="12765" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="30240" windowHeight="17900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Example Effects Table" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="639" uniqueCount="201">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="639" uniqueCount="200">
   <si>
     <t>Factor</t>
   </si>
@@ -651,10 +651,6 @@
   </si>
   <si>
     <t>Risk 3</t>
-  </si>
-  <si>
-    <t>Risk 3</t>
-    <phoneticPr fontId="5" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -662,13 +658,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="176" formatCode="0.000"/>
+    <numFmt numFmtId="164" formatCode="0.000"/>
   </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="等线"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -676,7 +672,7 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="等线"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -684,35 +680,28 @@
       <b/>
       <sz val="12"/>
       <color theme="1"/>
-      <name val="等线"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="12"/>
       <color theme="1"/>
-      <name val="等线"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="12"/>
       <color rgb="FF333333"/>
-      <name val="等线"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="8"/>
-      <name val="等线"/>
+      <name val="Calibri"/>
       <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <name val="等线"/>
-      <family val="3"/>
-      <charset val="134"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -883,7 +872,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="176" fontId="3" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -900,14 +889,14 @@
     <xf numFmtId="0" fontId="0" fillId="13" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="176" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="176" fontId="0" fillId="13" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="176" fontId="0" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="176" fontId="0" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="176" fontId="0" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="13" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="常规" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1186,24 +1175,24 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AY25"/>
-  <sheetFormatPr defaultColWidth="8.73046875" defaultRowHeight="13.9" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="22.19921875" customWidth="1"/>
-    <col min="3" max="3" width="20.796875" customWidth="1"/>
-    <col min="4" max="4" width="26.46484375" customWidth="1"/>
-    <col min="5" max="5" width="14.73046875" customWidth="1"/>
-    <col min="6" max="6" width="10.53125" customWidth="1"/>
-    <col min="7" max="7" width="12.265625" customWidth="1"/>
-    <col min="15" max="15" width="9.19921875" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="11.796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.1640625" customWidth="1"/>
+    <col min="3" max="3" width="20.83203125" customWidth="1"/>
+    <col min="4" max="4" width="26.5" customWidth="1"/>
+    <col min="5" max="5" width="14.6640625" customWidth="1"/>
+    <col min="6" max="6" width="10.5" customWidth="1"/>
+    <col min="7" max="7" width="12.33203125" customWidth="1"/>
+    <col min="15" max="15" width="9.1640625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="11.83203125" bestFit="1" customWidth="1"/>
     <col min="22" max="22" width="12" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="10.265625" customWidth="1"/>
-    <col min="24" max="24" width="9.19921875" customWidth="1"/>
-    <col min="29" max="29" width="9.19921875" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="11.796875" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="10.33203125" customWidth="1"/>
+    <col min="24" max="24" width="9.1640625" customWidth="1"/>
+    <col min="29" max="29" width="9.1640625" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="11.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:51" s="23" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:51" s="23" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="24" t="s">
         <v>0</v>
       </c>
@@ -1358,7 +1347,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="2" spans="1:51" s="23" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:51" s="23" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A2" s="23" t="s">
         <v>49</v>
       </c>
@@ -1434,7 +1423,7 @@
       <c r="AI2" s="33"/>
       <c r="AJ2" s="33"/>
     </row>
-    <row r="3" spans="1:51" s="23" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:51" s="23" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A3" s="23" t="s">
         <v>49</v>
       </c>
@@ -1478,11 +1467,11 @@
       <c r="R3" s="33"/>
       <c r="S3" s="33"/>
       <c r="T3" s="34">
-        <v>65</v>
+        <v>20</v>
       </c>
       <c r="U3" s="34"/>
       <c r="V3" s="34">
-        <v>63</v>
+        <v>16</v>
       </c>
       <c r="W3" s="23" t="s">
         <v>55</v>
@@ -1499,14 +1488,14 @@
       <c r="AF3" s="33"/>
       <c r="AG3" s="33"/>
       <c r="AH3" s="34">
-        <v>20</v>
+        <v>65</v>
       </c>
       <c r="AI3" s="34"/>
       <c r="AJ3" s="34">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="4" spans="1:51" s="23" customFormat="1" x14ac:dyDescent="0.4">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="4" spans="1:51" s="23" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A4" s="23" t="s">
         <v>49</v>
       </c>
@@ -1575,7 +1564,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:51" s="23" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:51" s="23" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A5" s="23" t="s">
         <v>61</v>
       </c>
@@ -1667,7 +1656,7 @@
       <c r="AI5" s="33"/>
       <c r="AJ5" s="33"/>
     </row>
-    <row r="6" spans="1:51" s="23" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:51" s="23" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A6" s="23" t="s">
         <v>61</v>
       </c>
@@ -1756,7 +1745,7 @@
       <c r="AI6" s="33"/>
       <c r="AJ6" s="33"/>
     </row>
-    <row r="7" spans="1:51" s="23" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:51" s="23" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A7" s="23" t="s">
         <v>61</v>
       </c>
@@ -1846,7 +1835,7 @@
       <c r="AI7" s="33"/>
       <c r="AJ7" s="33"/>
     </row>
-    <row r="8" spans="1:51" s="30" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:51" s="30" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A8" s="30" t="s">
         <v>49</v>
       </c>
@@ -1922,7 +1911,7 @@
       <c r="AI8" s="33"/>
       <c r="AJ8" s="33"/>
     </row>
-    <row r="9" spans="1:51" s="30" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:51" s="30" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A9" s="30" t="s">
         <v>49</v>
       </c>
@@ -1991,7 +1980,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="10" spans="1:51" s="30" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:51" s="30" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A10" s="30" t="s">
         <v>49</v>
       </c>
@@ -2062,7 +2051,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="11" spans="1:51" s="30" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:51" s="30" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A11" s="30" t="s">
         <v>61</v>
       </c>
@@ -2154,7 +2143,7 @@
       <c r="AI11" s="33"/>
       <c r="AJ11" s="33"/>
     </row>
-    <row r="12" spans="1:51" s="30" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:51" s="30" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A12" s="30" t="s">
         <v>61</v>
       </c>
@@ -2244,7 +2233,7 @@
       <c r="AI12" s="33"/>
       <c r="AJ12" s="33"/>
     </row>
-    <row r="13" spans="1:51" s="30" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:51" s="30" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A13" s="30" t="s">
         <v>61</v>
       </c>
@@ -2252,7 +2241,7 @@
         <v>175</v>
       </c>
       <c r="C13" s="30" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="D13" s="30" t="s">
         <v>178</v>
@@ -2334,7 +2323,7 @@
       <c r="AI13" s="33"/>
       <c r="AJ13" s="33"/>
     </row>
-    <row r="14" spans="1:51" s="31" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:51" s="31" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A14" s="31" t="s">
         <v>49</v>
       </c>
@@ -2410,7 +2399,7 @@
       <c r="AI14" s="33"/>
       <c r="AJ14" s="33"/>
     </row>
-    <row r="15" spans="1:51" s="31" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:51" s="31" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A15" s="31" t="s">
         <v>49</v>
       </c>
@@ -2479,7 +2468,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="16" spans="1:51" s="31" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:51" s="31" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A16" s="31" t="s">
         <v>49</v>
       </c>
@@ -2550,7 +2539,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="17" spans="1:36" s="31" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:36" s="31" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A17" s="31" t="s">
         <v>61</v>
       </c>
@@ -2642,7 +2631,7 @@
       <c r="AI17" s="33"/>
       <c r="AJ17" s="33"/>
     </row>
-    <row r="18" spans="1:36" s="31" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:36" s="31" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A18" s="31" t="s">
         <v>61</v>
       </c>
@@ -2732,7 +2721,7 @@
       <c r="AI18" s="33"/>
       <c r="AJ18" s="33"/>
     </row>
-    <row r="19" spans="1:36" s="31" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:36" s="31" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A19" s="31" t="s">
         <v>61</v>
       </c>
@@ -2822,7 +2811,7 @@
       <c r="AI19" s="33"/>
       <c r="AJ19" s="33"/>
     </row>
-    <row r="20" spans="1:36" s="32" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:36" s="32" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A20" s="32" t="s">
         <v>49</v>
       </c>
@@ -2898,7 +2887,7 @@
       <c r="AI20" s="33"/>
       <c r="AJ20" s="33"/>
     </row>
-    <row r="21" spans="1:36" s="32" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:36" s="32" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A21" s="32" t="s">
         <v>49</v>
       </c>
@@ -2977,7 +2966,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="22" spans="1:36" s="32" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:36" s="32" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A22" s="32" t="s">
         <v>49</v>
       </c>
@@ -3049,7 +3038,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="23" spans="1:36" s="32" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:36" s="32" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A23" s="32" t="s">
         <v>61</v>
       </c>
@@ -3142,7 +3131,7 @@
       <c r="AI23" s="33"/>
       <c r="AJ23" s="33"/>
     </row>
-    <row r="24" spans="1:36" s="32" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:36" s="32" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A24" s="32" t="s">
         <v>61</v>
       </c>
@@ -3232,7 +3221,7 @@
       <c r="AI24" s="33"/>
       <c r="AJ24" s="33"/>
     </row>
-    <row r="25" spans="1:36" s="32" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:36" s="32" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A25" s="32" t="s">
         <v>61</v>
       </c>
@@ -3332,14 +3321,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5D4A282F-FA68-4BC3-9814-08A63A8C35E3}">
   <dimension ref="A1:C16"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="16.46484375" style="16" customWidth="1"/>
-    <col min="2" max="2" width="7.19921875" style="16" customWidth="1"/>
-    <col min="3" max="3" width="12.265625" style="17" customWidth="1"/>
+    <col min="1" max="1" width="16.5" style="16" customWidth="1"/>
+    <col min="2" max="2" width="7.1640625" style="16" customWidth="1"/>
+    <col min="3" max="3" width="12.33203125" style="17" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" s="15" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" s="15" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="18" t="s">
         <v>179</v>
       </c>
@@ -3350,7 +3339,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" s="20" t="s">
         <v>182</v>
       </c>
@@ -3361,7 +3350,7 @@
         <v>0.02</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" s="20" t="s">
         <v>182</v>
       </c>
@@ -3372,7 +3361,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" s="20" t="s">
         <v>182</v>
       </c>
@@ -3383,7 +3372,7 @@
         <v>0.25</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" s="20" t="s">
         <v>181</v>
       </c>
@@ -3394,7 +3383,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" s="20" t="s">
         <v>181</v>
       </c>
@@ -3405,7 +3394,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" s="20" t="s">
         <v>181</v>
       </c>
@@ -3416,7 +3405,7 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" s="20" t="s">
         <v>183</v>
       </c>
@@ -3427,7 +3416,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A9" s="20" t="s">
         <v>183</v>
       </c>
@@ -3438,7 +3427,7 @@
         <v>0.25</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A10" s="20" t="s">
         <v>183</v>
       </c>
@@ -3449,7 +3438,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A11" s="22" t="s">
         <v>184</v>
       </c>
@@ -3460,7 +3449,7 @@
         <v>1E-3</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A12" s="20" t="s">
         <v>184</v>
       </c>
@@ -3471,7 +3460,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A13" s="20" t="s">
         <v>184</v>
       </c>
@@ -3482,7 +3471,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A14" s="20" t="s">
         <v>185</v>
       </c>
@@ -3493,7 +3482,7 @@
         <v>1E-3</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A15" s="20" t="s">
         <v>185</v>
       </c>
@@ -3504,7 +3493,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A16" s="20" t="s">
         <v>185</v>
       </c>
@@ -3516,7 +3505,6 @@
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="6" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -3524,18 +3512,18 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F7B77BDC-7246-43E5-B2E5-9DD908E43155}">
   <dimension ref="A1:G60"/>
-  <sheetFormatPr defaultRowHeight="13.9" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="17.46484375" style="13" customWidth="1"/>
-    <col min="2" max="2" width="21.796875" style="13" customWidth="1"/>
-    <col min="3" max="3" width="42.53125" style="13" customWidth="1"/>
-    <col min="4" max="4" width="9.73046875" style="14" customWidth="1"/>
+    <col min="1" max="1" width="17.5" style="13" customWidth="1"/>
+    <col min="2" max="2" width="21.83203125" style="13" customWidth="1"/>
+    <col min="3" max="3" width="42.5" style="13" customWidth="1"/>
+    <col min="4" max="4" width="9.6640625" style="14" customWidth="1"/>
     <col min="5" max="5" width="18" style="13" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="22.53125" style="13" customWidth="1"/>
-    <col min="7" max="7" width="35.265625" style="14" customWidth="1"/>
+    <col min="6" max="6" width="22.5" style="13" customWidth="1"/>
+    <col min="7" max="7" width="35.33203125" style="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" s="1" customFormat="1" ht="97.15" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:7" s="1" customFormat="1" ht="96" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>170</v>
       </c>
@@ -3558,7 +3546,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A2" s="3" t="s">
         <v>0</v>
       </c>
@@ -3577,7 +3565,7 @@
       <c r="F2" s="3"/>
       <c r="G2" s="4"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
@@ -3596,7 +3584,7 @@
       </c>
       <c r="G3" s="4"/>
     </row>
-    <row r="4" spans="1:7" ht="41.65" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:7" ht="48" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -3615,7 +3603,7 @@
       </c>
       <c r="G4" s="4"/>
     </row>
-    <row r="5" spans="1:7" ht="27.75" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:7" ht="32" x14ac:dyDescent="0.2">
       <c r="A5" s="3" t="s">
         <v>3</v>
       </c>
@@ -3634,7 +3622,7 @@
       </c>
       <c r="G5" s="4"/>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A6" s="3" t="s">
         <v>4</v>
       </c>
@@ -3653,7 +3641,7 @@
       <c r="F6" s="3"/>
       <c r="G6" s="4"/>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A7" s="3" t="s">
         <v>6</v>
       </c>
@@ -3672,7 +3660,7 @@
       <c r="F7" s="3"/>
       <c r="G7" s="4"/>
     </row>
-    <row r="8" spans="1:7" ht="27.75" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:7" ht="32" x14ac:dyDescent="0.2">
       <c r="A8" s="3" t="s">
         <v>7</v>
       </c>
@@ -3693,7 +3681,7 @@
       </c>
       <c r="G8" s="4"/>
     </row>
-    <row r="9" spans="1:7" ht="27.75" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:7" ht="32" x14ac:dyDescent="0.2">
       <c r="A9" s="3" t="s">
         <v>8</v>
       </c>
@@ -3714,7 +3702,7 @@
       </c>
       <c r="G9" s="4"/>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A10" s="3" t="s">
         <v>9</v>
       </c>
@@ -3733,7 +3721,7 @@
       </c>
       <c r="G10" s="4"/>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A11" s="3" t="s">
         <v>23</v>
       </c>
@@ -3752,7 +3740,7 @@
       <c r="F11" s="3"/>
       <c r="G11" s="4"/>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A12" s="3" t="s">
         <v>22</v>
       </c>
@@ -3771,7 +3759,7 @@
       <c r="F12" s="3"/>
       <c r="G12" s="4"/>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" s="3"/>
       <c r="B13" s="3"/>
       <c r="C13" s="3"/>
@@ -3780,7 +3768,7 @@
       <c r="F13" s="3"/>
       <c r="G13" s="4"/>
     </row>
-    <row r="14" spans="1:7" ht="97.15" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:7" ht="96" x14ac:dyDescent="0.2">
       <c r="A14" s="5" t="s">
         <v>169</v>
       </c>
@@ -3803,7 +3791,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="15" spans="1:7" ht="27.75" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:7" ht="32" x14ac:dyDescent="0.2">
       <c r="A15" s="3" t="s">
         <v>5</v>
       </c>
@@ -3822,7 +3810,7 @@
       <c r="F15" s="3"/>
       <c r="G15" s="4"/>
     </row>
-    <row r="16" spans="1:7" ht="41.65" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:7" ht="48" x14ac:dyDescent="0.2">
       <c r="A16" s="3" t="s">
         <v>12</v>
       </c>
@@ -3839,7 +3827,7 @@
       <c r="F16" s="3"/>
       <c r="G16" s="4"/>
     </row>
-    <row r="17" spans="1:7" ht="55.5" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:7" ht="64" x14ac:dyDescent="0.2">
       <c r="A17" s="3" t="s">
         <v>15</v>
       </c>
@@ -3856,7 +3844,7 @@
       <c r="F17" s="3"/>
       <c r="G17" s="4"/>
     </row>
-    <row r="18" spans="1:7" ht="55.5" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:7" ht="64" x14ac:dyDescent="0.2">
       <c r="A18" s="3" t="s">
         <v>18</v>
       </c>
@@ -3873,7 +3861,7 @@
       <c r="F18" s="3"/>
       <c r="G18" s="4"/>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A19" s="3" t="s">
         <v>19</v>
       </c>
@@ -3890,7 +3878,7 @@
       <c r="F19" s="3"/>
       <c r="G19" s="4"/>
     </row>
-    <row r="20" spans="1:7" ht="41.65" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:7" ht="48" x14ac:dyDescent="0.2">
       <c r="A20" s="3" t="s">
         <v>26</v>
       </c>
@@ -3907,7 +3895,7 @@
       <c r="F20" s="3"/>
       <c r="G20" s="4"/>
     </row>
-    <row r="21" spans="1:7" ht="55.5" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:7" ht="64" x14ac:dyDescent="0.2">
       <c r="A21" s="3" t="s">
         <v>29</v>
       </c>
@@ -3924,7 +3912,7 @@
       <c r="F21" s="3"/>
       <c r="G21" s="4"/>
     </row>
-    <row r="22" spans="1:7" ht="55.5" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:7" ht="64" x14ac:dyDescent="0.2">
       <c r="A22" s="3" t="s">
         <v>32</v>
       </c>
@@ -3941,7 +3929,7 @@
       <c r="F22" s="3"/>
       <c r="G22" s="4"/>
     </row>
-    <row r="23" spans="1:7" ht="27.75" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:7" ht="32" x14ac:dyDescent="0.2">
       <c r="A23" s="3" t="s">
         <v>33</v>
       </c>
@@ -3958,7 +3946,7 @@
       <c r="F23" s="3"/>
       <c r="G23" s="4"/>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A24" s="3"/>
       <c r="B24" s="3"/>
       <c r="C24" s="3"/>
@@ -3967,7 +3955,7 @@
       <c r="F24" s="3"/>
       <c r="G24" s="4"/>
     </row>
-    <row r="25" spans="1:7" ht="83.25" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:7" ht="80" x14ac:dyDescent="0.2">
       <c r="A25" s="7" t="s">
         <v>171</v>
       </c>
@@ -3990,7 +3978,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="26" spans="1:7" ht="27.75" x14ac:dyDescent="0.4">
+    <row r="26" spans="1:7" ht="32" x14ac:dyDescent="0.2">
       <c r="A26" s="3" t="s">
         <v>11</v>
       </c>
@@ -4007,7 +3995,7 @@
       <c r="F26" s="3"/>
       <c r="G26" s="4"/>
     </row>
-    <row r="27" spans="1:7" ht="41.65" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:7" ht="48" x14ac:dyDescent="0.2">
       <c r="A27" s="3" t="s">
         <v>14</v>
       </c>
@@ -4024,7 +4012,7 @@
       <c r="F27" s="3"/>
       <c r="G27" s="4"/>
     </row>
-    <row r="28" spans="1:7" ht="41.65" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:7" ht="48" x14ac:dyDescent="0.2">
       <c r="A28" s="3" t="s">
         <v>17</v>
       </c>
@@ -4041,7 +4029,7 @@
       <c r="F28" s="3"/>
       <c r="G28" s="4"/>
     </row>
-    <row r="29" spans="1:7" ht="55.5" x14ac:dyDescent="0.4">
+    <row r="29" spans="1:7" ht="64" x14ac:dyDescent="0.2">
       <c r="A29" s="3" t="s">
         <v>21</v>
       </c>
@@ -4058,7 +4046,7 @@
       <c r="F29" s="3"/>
       <c r="G29" s="4"/>
     </row>
-    <row r="30" spans="1:7" ht="27.75" x14ac:dyDescent="0.4">
+    <row r="30" spans="1:7" ht="32" x14ac:dyDescent="0.2">
       <c r="A30" s="3" t="s">
         <v>25</v>
       </c>
@@ -4075,7 +4063,7 @@
       <c r="F30" s="3"/>
       <c r="G30" s="4"/>
     </row>
-    <row r="31" spans="1:7" ht="41.65" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:7" ht="48" x14ac:dyDescent="0.2">
       <c r="A31" s="3" t="s">
         <v>28</v>
       </c>
@@ -4092,7 +4080,7 @@
       <c r="F31" s="3"/>
       <c r="G31" s="4"/>
     </row>
-    <row r="32" spans="1:7" ht="41.65" x14ac:dyDescent="0.4">
+    <row r="32" spans="1:7" ht="48" x14ac:dyDescent="0.2">
       <c r="A32" s="3" t="s">
         <v>31</v>
       </c>
@@ -4109,7 +4097,7 @@
       <c r="F32" s="3"/>
       <c r="G32" s="4"/>
     </row>
-    <row r="33" spans="1:7" ht="55.5" x14ac:dyDescent="0.4">
+    <row r="33" spans="1:7" ht="64" x14ac:dyDescent="0.2">
       <c r="A33" s="3" t="s">
         <v>35</v>
       </c>
@@ -4126,7 +4114,7 @@
       <c r="F33" s="3"/>
       <c r="G33" s="4"/>
     </row>
-    <row r="34" spans="1:7" ht="111" x14ac:dyDescent="0.4">
+    <row r="34" spans="1:7" ht="128" x14ac:dyDescent="0.2">
       <c r="A34" s="3" t="s">
         <v>36</v>
       </c>
@@ -4145,7 +4133,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="35" spans="1:7" ht="111" x14ac:dyDescent="0.4">
+    <row r="35" spans="1:7" ht="128" x14ac:dyDescent="0.2">
       <c r="A35" s="3" t="s">
         <v>37</v>
       </c>
@@ -4164,7 +4152,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="36" spans="1:7" ht="55.5" x14ac:dyDescent="0.4">
+    <row r="36" spans="1:7" ht="48" x14ac:dyDescent="0.2">
       <c r="A36" s="3" t="s">
         <v>38</v>
       </c>
@@ -4183,7 +4171,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="37" spans="1:7" ht="55.5" x14ac:dyDescent="0.4">
+    <row r="37" spans="1:7" ht="48" x14ac:dyDescent="0.2">
       <c r="A37" s="3" t="s">
         <v>39</v>
       </c>
@@ -4202,7 +4190,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="38" spans="1:7" ht="55.5" x14ac:dyDescent="0.4">
+    <row r="38" spans="1:7" ht="48" x14ac:dyDescent="0.2">
       <c r="A38" s="3" t="s">
         <v>162</v>
       </c>
@@ -4221,7 +4209,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="39" spans="1:7" ht="55.5" x14ac:dyDescent="0.4">
+    <row r="39" spans="1:7" ht="48" x14ac:dyDescent="0.2">
       <c r="A39" s="3" t="s">
         <v>163</v>
       </c>
@@ -4240,7 +4228,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="40" spans="1:7" ht="55.5" x14ac:dyDescent="0.4">
+    <row r="40" spans="1:7" ht="64" x14ac:dyDescent="0.2">
       <c r="A40" s="3" t="s">
         <v>40</v>
       </c>
@@ -4259,7 +4247,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="41" spans="1:7" ht="55.5" x14ac:dyDescent="0.4">
+    <row r="41" spans="1:7" ht="64" x14ac:dyDescent="0.2">
       <c r="A41" s="3" t="s">
         <v>41</v>
       </c>
@@ -4278,7 +4266,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="42" spans="1:7" ht="83.25" x14ac:dyDescent="0.4">
+    <row r="42" spans="1:7" ht="80" x14ac:dyDescent="0.2">
       <c r="A42" s="3" t="s">
         <v>42</v>
       </c>
@@ -4297,7 +4285,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="43" spans="1:7" ht="83.25" x14ac:dyDescent="0.4">
+    <row r="43" spans="1:7" ht="80" x14ac:dyDescent="0.2">
       <c r="A43" s="3" t="s">
         <v>43</v>
       </c>
@@ -4316,7 +4304,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A44" s="3"/>
       <c r="B44" s="3"/>
       <c r="C44" s="3"/>
@@ -4325,7 +4313,7 @@
       <c r="F44" s="3"/>
       <c r="G44" s="4"/>
     </row>
-    <row r="45" spans="1:7" ht="83.25" x14ac:dyDescent="0.4">
+    <row r="45" spans="1:7" ht="96" x14ac:dyDescent="0.2">
       <c r="A45" s="9" t="s">
         <v>172</v>
       </c>
@@ -4348,7 +4336,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="46" spans="1:7" ht="41.65" x14ac:dyDescent="0.4">
+    <row r="46" spans="1:7" ht="32" x14ac:dyDescent="0.2">
       <c r="A46" s="3" t="s">
         <v>10</v>
       </c>
@@ -4365,7 +4353,7 @@
       <c r="F46" s="3"/>
       <c r="G46" s="4"/>
     </row>
-    <row r="47" spans="1:7" ht="27.75" x14ac:dyDescent="0.4">
+    <row r="47" spans="1:7" ht="32" x14ac:dyDescent="0.2">
       <c r="A47" s="3" t="s">
         <v>13</v>
       </c>
@@ -4382,7 +4370,7 @@
       <c r="F47" s="3"/>
       <c r="G47" s="4"/>
     </row>
-    <row r="48" spans="1:7" ht="27.75" x14ac:dyDescent="0.4">
+    <row r="48" spans="1:7" ht="32" x14ac:dyDescent="0.2">
       <c r="A48" s="3" t="s">
         <v>16</v>
       </c>
@@ -4399,7 +4387,7 @@
       <c r="F48" s="3"/>
       <c r="G48" s="4"/>
     </row>
-    <row r="49" spans="1:7" ht="27.75" x14ac:dyDescent="0.4">
+    <row r="49" spans="1:7" ht="32" x14ac:dyDescent="0.2">
       <c r="A49" s="3" t="s">
         <v>20</v>
       </c>
@@ -4416,7 +4404,7 @@
       <c r="F49" s="3"/>
       <c r="G49" s="4"/>
     </row>
-    <row r="50" spans="1:7" ht="41.65" x14ac:dyDescent="0.4">
+    <row r="50" spans="1:7" ht="48" x14ac:dyDescent="0.2">
       <c r="A50" s="3" t="s">
         <v>24</v>
       </c>
@@ -4433,7 +4421,7 @@
       <c r="F50" s="3"/>
       <c r="G50" s="4"/>
     </row>
-    <row r="51" spans="1:7" ht="27.75" x14ac:dyDescent="0.4">
+    <row r="51" spans="1:7" ht="32" x14ac:dyDescent="0.2">
       <c r="A51" s="3" t="s">
         <v>27</v>
       </c>
@@ -4450,7 +4438,7 @@
       <c r="F51" s="3"/>
       <c r="G51" s="4"/>
     </row>
-    <row r="52" spans="1:7" ht="27.75" x14ac:dyDescent="0.4">
+    <row r="52" spans="1:7" ht="32" x14ac:dyDescent="0.2">
       <c r="A52" s="3" t="s">
         <v>30</v>
       </c>
@@ -4467,7 +4455,7 @@
       <c r="F52" s="3"/>
       <c r="G52" s="4"/>
     </row>
-    <row r="53" spans="1:7" ht="27.75" x14ac:dyDescent="0.4">
+    <row r="53" spans="1:7" ht="32" x14ac:dyDescent="0.2">
       <c r="A53" s="3" t="s">
         <v>34</v>
       </c>
@@ -4484,7 +4472,7 @@
       <c r="F53" s="3"/>
       <c r="G53" s="4"/>
     </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="54" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A54" s="3"/>
       <c r="B54" s="3"/>
       <c r="C54" s="3"/>
@@ -4493,7 +4481,7 @@
       <c r="F54" s="3"/>
       <c r="G54" s="4"/>
     </row>
-    <row r="55" spans="1:7" ht="69.400000000000006" x14ac:dyDescent="0.4">
+    <row r="55" spans="1:7" ht="64" x14ac:dyDescent="0.2">
       <c r="A55" s="11" t="s">
         <v>173</v>
       </c>
@@ -4516,7 +4504,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="56" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A56" s="3" t="s">
         <v>44</v>
       </c>
@@ -4533,7 +4521,7 @@
       <c r="F56" s="3"/>
       <c r="G56" s="4"/>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="57" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A57" s="3" t="s">
         <v>45</v>
       </c>
@@ -4552,7 +4540,7 @@
       </c>
       <c r="G57" s="4"/>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="58" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A58" s="3" t="s">
         <v>46</v>
       </c>
@@ -4571,7 +4559,7 @@
       </c>
       <c r="G58" s="4"/>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="59" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A59" s="3" t="s">
         <v>47</v>
       </c>
@@ -4588,7 +4576,7 @@
       <c r="F59" s="3"/>
       <c r="G59" s="4"/>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="60" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A60" s="3" t="s">
         <v>48</v>
       </c>
@@ -4606,32 +4594,11 @@
       <c r="G60" s="4"/>
     </row>
   </sheetData>
-  <phoneticPr fontId="6" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="e522a4ea-6824-496f-8ffe-e074cc291ac0">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="8080ce30-d5ea-40e8-a48f-b77958a33e4e" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100CBEA71EDBDE86541B7589EDD610CDCA6" ma:contentTypeVersion="10" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="6135c02e9fba22fa14c95532ff73e585">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="e522a4ea-6824-496f-8ffe-e074cc291ac0" xmlns:ns3="8080ce30-d5ea-40e8-a48f-b77958a33e4e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4c9beda59bcc2e0dae0951e4601e1985" ns2:_="" ns3:_="">
     <xsd:import namespace="e522a4ea-6824-496f-8ffe-e074cc291ac0"/>
@@ -4822,7 +4789,46 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="e522a4ea-6824-496f-8ffe-e074cc291ac0">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="8080ce30-d5ea-40e8-a48f-b77958a33e4e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EF3A5692-B908-4374-9724-9509DDA5EAF8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="e522a4ea-6824-496f-8ffe-e074cc291ac0"/>
+    <ds:schemaRef ds:uri="8080ce30-d5ea-40e8-a48f-b77958a33e4e"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{13FE4927-61BE-41A1-B367-1B1C5D848E2B}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
@@ -4839,7 +4845,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8E8BB74B-0686-4136-81AA-6AA3532E32A8}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
@@ -4847,21 +4853,8 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EF3A5692-B908-4374-9724-9509DDA5EAF8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="e522a4ea-6824-496f-8ffe-e074cc291ac0"/>
-    <ds:schemaRef ds:uri="8080ce30-d5ea-40e8-a48f-b77958a33e4e"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{f743b317-4758-44cb-8b65-8b43e4619766}" enabled="1" method="Standard" siteId="{fdfed7bd-9f6a-44a1-b694-6e39c468c150}" contentBits="0" removed="0"/>
+</clbl:labelList>
 </file>
</xml_diff>

<commit_message>
Synchronized with master branch
</commit_message>
<xml_diff>
--- a/data-raw/Manuscript_Generic_Example.xlsx
+++ b/data-raw/Manuscript_Generic_Example.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28925"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lgaka\Downloads\brpubVJCE\data-raw\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fengh\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45E440DB-7E6D-4DAC-9237-F4DD7BC63BA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7EF72D8-26E5-477D-81E3-22566F9AF6AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1470" yWindow="735" windowWidth="19793" windowHeight="12765" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Example Effects Table" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="639" uniqueCount="200">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="639" uniqueCount="201">
   <si>
     <t>Factor</t>
   </si>
@@ -651,6 +651,10 @@
   </si>
   <si>
     <t>Risk 3</t>
+  </si>
+  <si>
+    <t>Risk 3</t>
+    <phoneticPr fontId="5" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -658,13 +662,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="0.000"/>
+    <numFmt numFmtId="176" formatCode="0.000"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="等线"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -672,7 +676,7 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="等线"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -680,28 +684,35 @@
       <b/>
       <sz val="12"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="等线"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="12"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="等线"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="12"/>
       <color rgb="FF333333"/>
-      <name val="Calibri"/>
+      <name val="等线"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="8"/>
-      <name val="Calibri"/>
+      <name val="等线"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="等线"/>
+      <family val="3"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -872,7 +883,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="3" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="176" fontId="3" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -889,14 +900,14 @@
     <xf numFmtId="0" fontId="0" fillId="13" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="13" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="176" fontId="0" fillId="13" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="176" fontId="0" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="176" fontId="0" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="176" fontId="0" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="常规" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1175,24 +1186,24 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AY25"/>
-  <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.73046875" defaultRowHeight="13.9" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="2" max="2" width="22.1796875" customWidth="1"/>
-    <col min="3" max="3" width="20.81640625" customWidth="1"/>
-    <col min="4" max="4" width="26.453125" customWidth="1"/>
-    <col min="5" max="5" width="14.7265625" customWidth="1"/>
-    <col min="6" max="6" width="10.54296875" customWidth="1"/>
-    <col min="7" max="7" width="12.26953125" customWidth="1"/>
-    <col min="15" max="15" width="9.1796875" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="11.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.19921875" customWidth="1"/>
+    <col min="3" max="3" width="20.796875" customWidth="1"/>
+    <col min="4" max="4" width="26.46484375" customWidth="1"/>
+    <col min="5" max="5" width="14.73046875" customWidth="1"/>
+    <col min="6" max="6" width="10.53125" customWidth="1"/>
+    <col min="7" max="7" width="12.265625" customWidth="1"/>
+    <col min="15" max="15" width="9.19921875" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="11.796875" bestFit="1" customWidth="1"/>
     <col min="22" max="22" width="12" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="10.26953125" customWidth="1"/>
-    <col min="24" max="24" width="9.1796875" customWidth="1"/>
-    <col min="29" max="29" width="9.1796875" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="11.81640625" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="10.265625" customWidth="1"/>
+    <col min="24" max="24" width="9.19921875" customWidth="1"/>
+    <col min="29" max="29" width="9.19921875" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="11.796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:51" s="23" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:51" s="23" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A1" s="24" t="s">
         <v>0</v>
       </c>
@@ -1347,7 +1358,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="2" spans="1:51" s="23" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:51" s="23" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A2" s="23" t="s">
         <v>49</v>
       </c>
@@ -1423,7 +1434,7 @@
       <c r="AI2" s="33"/>
       <c r="AJ2" s="33"/>
     </row>
-    <row r="3" spans="1:51" s="23" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:51" s="23" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A3" s="23" t="s">
         <v>49</v>
       </c>
@@ -1495,7 +1506,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:51" s="23" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:51" s="23" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A4" s="23" t="s">
         <v>49</v>
       </c>
@@ -1564,7 +1575,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:51" s="23" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:51" s="23" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A5" s="23" t="s">
         <v>61</v>
       </c>
@@ -1656,7 +1667,7 @@
       <c r="AI5" s="33"/>
       <c r="AJ5" s="33"/>
     </row>
-    <row r="6" spans="1:51" s="23" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:51" s="23" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A6" s="23" t="s">
         <v>61</v>
       </c>
@@ -1745,7 +1756,7 @@
       <c r="AI6" s="33"/>
       <c r="AJ6" s="33"/>
     </row>
-    <row r="7" spans="1:51" s="23" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:51" s="23" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A7" s="23" t="s">
         <v>61</v>
       </c>
@@ -1835,7 +1846,7 @@
       <c r="AI7" s="33"/>
       <c r="AJ7" s="33"/>
     </row>
-    <row r="8" spans="1:51" s="30" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:51" s="30" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A8" s="30" t="s">
         <v>49</v>
       </c>
@@ -1911,7 +1922,7 @@
       <c r="AI8" s="33"/>
       <c r="AJ8" s="33"/>
     </row>
-    <row r="9" spans="1:51" s="30" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:51" s="30" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A9" s="30" t="s">
         <v>49</v>
       </c>
@@ -1980,7 +1991,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="10" spans="1:51" s="30" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:51" s="30" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A10" s="30" t="s">
         <v>49</v>
       </c>
@@ -2051,7 +2062,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="11" spans="1:51" s="30" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:51" s="30" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A11" s="30" t="s">
         <v>61</v>
       </c>
@@ -2143,7 +2154,7 @@
       <c r="AI11" s="33"/>
       <c r="AJ11" s="33"/>
     </row>
-    <row r="12" spans="1:51" s="30" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:51" s="30" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A12" s="30" t="s">
         <v>61</v>
       </c>
@@ -2233,7 +2244,7 @@
       <c r="AI12" s="33"/>
       <c r="AJ12" s="33"/>
     </row>
-    <row r="13" spans="1:51" s="30" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:51" s="30" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A13" s="30" t="s">
         <v>61</v>
       </c>
@@ -2241,7 +2252,7 @@
         <v>175</v>
       </c>
       <c r="C13" s="30" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="D13" s="30" t="s">
         <v>178</v>
@@ -2323,7 +2334,7 @@
       <c r="AI13" s="33"/>
       <c r="AJ13" s="33"/>
     </row>
-    <row r="14" spans="1:51" s="31" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:51" s="31" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A14" s="31" t="s">
         <v>49</v>
       </c>
@@ -2399,7 +2410,7 @@
       <c r="AI14" s="33"/>
       <c r="AJ14" s="33"/>
     </row>
-    <row r="15" spans="1:51" s="31" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:51" s="31" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A15" s="31" t="s">
         <v>49</v>
       </c>
@@ -2468,7 +2479,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="16" spans="1:51" s="31" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:51" s="31" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A16" s="31" t="s">
         <v>49</v>
       </c>
@@ -2539,7 +2550,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="17" spans="1:36" s="31" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:36" s="31" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A17" s="31" t="s">
         <v>61</v>
       </c>
@@ -2631,7 +2642,7 @@
       <c r="AI17" s="33"/>
       <c r="AJ17" s="33"/>
     </row>
-    <row r="18" spans="1:36" s="31" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:36" s="31" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A18" s="31" t="s">
         <v>61</v>
       </c>
@@ -2721,7 +2732,7 @@
       <c r="AI18" s="33"/>
       <c r="AJ18" s="33"/>
     </row>
-    <row r="19" spans="1:36" s="31" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:36" s="31" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A19" s="31" t="s">
         <v>61</v>
       </c>
@@ -2811,7 +2822,7 @@
       <c r="AI19" s="33"/>
       <c r="AJ19" s="33"/>
     </row>
-    <row r="20" spans="1:36" s="32" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:36" s="32" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A20" s="32" t="s">
         <v>49</v>
       </c>
@@ -2887,7 +2898,7 @@
       <c r="AI20" s="33"/>
       <c r="AJ20" s="33"/>
     </row>
-    <row r="21" spans="1:36" s="32" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:36" s="32" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A21" s="32" t="s">
         <v>49</v>
       </c>
@@ -2966,7 +2977,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="22" spans="1:36" s="32" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:36" s="32" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A22" s="32" t="s">
         <v>49</v>
       </c>
@@ -3038,7 +3049,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="23" spans="1:36" s="32" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:36" s="32" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A23" s="32" t="s">
         <v>61</v>
       </c>
@@ -3131,7 +3142,7 @@
       <c r="AI23" s="33"/>
       <c r="AJ23" s="33"/>
     </row>
-    <row r="24" spans="1:36" s="32" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:36" s="32" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A24" s="32" t="s">
         <v>61</v>
       </c>
@@ -3221,7 +3232,7 @@
       <c r="AI24" s="33"/>
       <c r="AJ24" s="33"/>
     </row>
-    <row r="25" spans="1:36" s="32" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:36" s="32" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A25" s="32" t="s">
         <v>61</v>
       </c>
@@ -3321,14 +3332,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5D4A282F-FA68-4BC3-9814-08A63A8C35E3}">
   <dimension ref="A1:C16"/>
-  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="16.453125" style="16" customWidth="1"/>
-    <col min="2" max="2" width="7.1796875" style="16" customWidth="1"/>
-    <col min="3" max="3" width="12.26953125" style="17" customWidth="1"/>
+    <col min="1" max="1" width="16.46484375" style="16" customWidth="1"/>
+    <col min="2" max="2" width="7.19921875" style="16" customWidth="1"/>
+    <col min="3" max="3" width="12.265625" style="17" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" s="15" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" s="15" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A1" s="18" t="s">
         <v>179</v>
       </c>
@@ -3339,7 +3350,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" s="20" t="s">
         <v>182</v>
       </c>
@@ -3350,7 +3361,7 @@
         <v>0.02</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" s="20" t="s">
         <v>182</v>
       </c>
@@ -3361,7 +3372,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" s="20" t="s">
         <v>182</v>
       </c>
@@ -3372,7 +3383,7 @@
         <v>0.25</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A5" s="20" t="s">
         <v>181</v>
       </c>
@@ -3383,7 +3394,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A6" s="20" t="s">
         <v>181</v>
       </c>
@@ -3394,7 +3405,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A7" s="20" t="s">
         <v>181</v>
       </c>
@@ -3405,7 +3416,7 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A8" s="20" t="s">
         <v>183</v>
       </c>
@@ -3416,7 +3427,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A9" s="20" t="s">
         <v>183</v>
       </c>
@@ -3427,7 +3438,7 @@
         <v>0.25</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A10" s="20" t="s">
         <v>183</v>
       </c>
@@ -3438,7 +3449,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A11" s="22" t="s">
         <v>184</v>
       </c>
@@ -3449,7 +3460,7 @@
         <v>1E-3</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A12" s="20" t="s">
         <v>184</v>
       </c>
@@ -3460,7 +3471,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A13" s="20" t="s">
         <v>184</v>
       </c>
@@ -3471,7 +3482,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A14" s="20" t="s">
         <v>185</v>
       </c>
@@ -3482,7 +3493,7 @@
         <v>1E-3</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A15" s="20" t="s">
         <v>185</v>
       </c>
@@ -3493,7 +3504,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A16" s="20" t="s">
         <v>185</v>
       </c>
@@ -3505,6 +3516,7 @@
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="6" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -3512,18 +3524,18 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F7B77BDC-7246-43E5-B2E5-9DD908E43155}">
   <dimension ref="A1:G60"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="13.9" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="17.453125" style="13" customWidth="1"/>
-    <col min="2" max="2" width="21.81640625" style="13" customWidth="1"/>
-    <col min="3" max="3" width="42.54296875" style="13" customWidth="1"/>
-    <col min="4" max="4" width="9.7265625" style="14" customWidth="1"/>
+    <col min="1" max="1" width="17.46484375" style="13" customWidth="1"/>
+    <col min="2" max="2" width="21.796875" style="13" customWidth="1"/>
+    <col min="3" max="3" width="42.53125" style="13" customWidth="1"/>
+    <col min="4" max="4" width="9.73046875" style="14" customWidth="1"/>
     <col min="5" max="5" width="18" style="13" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="22.54296875" style="13" customWidth="1"/>
-    <col min="7" max="7" width="35.26953125" style="14" customWidth="1"/>
+    <col min="6" max="6" width="22.53125" style="13" customWidth="1"/>
+    <col min="7" max="7" width="35.265625" style="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" s="1" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" s="1" customFormat="1" ht="97.15" x14ac:dyDescent="0.4">
       <c r="A1" s="2" t="s">
         <v>170</v>
       </c>
@@ -3546,7 +3558,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A2" s="3" t="s">
         <v>0</v>
       </c>
@@ -3565,7 +3577,7 @@
       <c r="F2" s="3"/>
       <c r="G2" s="4"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
@@ -3584,7 +3596,7 @@
       </c>
       <c r="G3" s="4"/>
     </row>
-    <row r="4" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:7" ht="41.65" x14ac:dyDescent="0.4">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -3603,7 +3615,7 @@
       </c>
       <c r="G4" s="4"/>
     </row>
-    <row r="5" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:7" ht="27.75" x14ac:dyDescent="0.4">
       <c r="A5" s="3" t="s">
         <v>3</v>
       </c>
@@ -3622,7 +3634,7 @@
       </c>
       <c r="G5" s="4"/>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A6" s="3" t="s">
         <v>4</v>
       </c>
@@ -3641,7 +3653,7 @@
       <c r="F6" s="3"/>
       <c r="G6" s="4"/>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A7" s="3" t="s">
         <v>6</v>
       </c>
@@ -3660,7 +3672,7 @@
       <c r="F7" s="3"/>
       <c r="G7" s="4"/>
     </row>
-    <row r="8" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:7" ht="27.75" x14ac:dyDescent="0.4">
       <c r="A8" s="3" t="s">
         <v>7</v>
       </c>
@@ -3681,7 +3693,7 @@
       </c>
       <c r="G8" s="4"/>
     </row>
-    <row r="9" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:7" ht="27.75" x14ac:dyDescent="0.4">
       <c r="A9" s="3" t="s">
         <v>8</v>
       </c>
@@ -3702,7 +3714,7 @@
       </c>
       <c r="G9" s="4"/>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A10" s="3" t="s">
         <v>9</v>
       </c>
@@ -3721,7 +3733,7 @@
       </c>
       <c r="G10" s="4"/>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A11" s="3" t="s">
         <v>23</v>
       </c>
@@ -3740,7 +3752,7 @@
       <c r="F11" s="3"/>
       <c r="G11" s="4"/>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A12" s="3" t="s">
         <v>22</v>
       </c>
@@ -3759,7 +3771,7 @@
       <c r="F12" s="3"/>
       <c r="G12" s="4"/>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A13" s="3"/>
       <c r="B13" s="3"/>
       <c r="C13" s="3"/>
@@ -3768,7 +3780,7 @@
       <c r="F13" s="3"/>
       <c r="G13" s="4"/>
     </row>
-    <row r="14" spans="1:7" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:7" ht="97.15" x14ac:dyDescent="0.4">
       <c r="A14" s="5" t="s">
         <v>169</v>
       </c>
@@ -3791,7 +3803,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="15" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:7" ht="27.75" x14ac:dyDescent="0.4">
       <c r="A15" s="3" t="s">
         <v>5</v>
       </c>
@@ -3810,7 +3822,7 @@
       <c r="F15" s="3"/>
       <c r="G15" s="4"/>
     </row>
-    <row r="16" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:7" ht="41.65" x14ac:dyDescent="0.4">
       <c r="A16" s="3" t="s">
         <v>12</v>
       </c>
@@ -3827,7 +3839,7 @@
       <c r="F16" s="3"/>
       <c r="G16" s="4"/>
     </row>
-    <row r="17" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:7" ht="55.5" x14ac:dyDescent="0.4">
       <c r="A17" s="3" t="s">
         <v>15</v>
       </c>
@@ -3844,7 +3856,7 @@
       <c r="F17" s="3"/>
       <c r="G17" s="4"/>
     </row>
-    <row r="18" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:7" ht="55.5" x14ac:dyDescent="0.4">
       <c r="A18" s="3" t="s">
         <v>18</v>
       </c>
@@ -3861,7 +3873,7 @@
       <c r="F18" s="3"/>
       <c r="G18" s="4"/>
     </row>
-    <row r="19" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A19" s="3" t="s">
         <v>19</v>
       </c>
@@ -3878,7 +3890,7 @@
       <c r="F19" s="3"/>
       <c r="G19" s="4"/>
     </row>
-    <row r="20" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:7" ht="41.65" x14ac:dyDescent="0.4">
       <c r="A20" s="3" t="s">
         <v>26</v>
       </c>
@@ -3895,7 +3907,7 @@
       <c r="F20" s="3"/>
       <c r="G20" s="4"/>
     </row>
-    <row r="21" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:7" ht="55.5" x14ac:dyDescent="0.4">
       <c r="A21" s="3" t="s">
         <v>29</v>
       </c>
@@ -3912,7 +3924,7 @@
       <c r="F21" s="3"/>
       <c r="G21" s="4"/>
     </row>
-    <row r="22" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:7" ht="55.5" x14ac:dyDescent="0.4">
       <c r="A22" s="3" t="s">
         <v>32</v>
       </c>
@@ -3929,7 +3941,7 @@
       <c r="F22" s="3"/>
       <c r="G22" s="4"/>
     </row>
-    <row r="23" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:7" ht="27.75" x14ac:dyDescent="0.4">
       <c r="A23" s="3" t="s">
         <v>33</v>
       </c>
@@ -3946,7 +3958,7 @@
       <c r="F23" s="3"/>
       <c r="G23" s="4"/>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A24" s="3"/>
       <c r="B24" s="3"/>
       <c r="C24" s="3"/>
@@ -3955,7 +3967,7 @@
       <c r="F24" s="3"/>
       <c r="G24" s="4"/>
     </row>
-    <row r="25" spans="1:7" ht="87" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:7" ht="83.25" x14ac:dyDescent="0.4">
       <c r="A25" s="7" t="s">
         <v>171</v>
       </c>
@@ -3978,7 +3990,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="26" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:7" ht="27.75" x14ac:dyDescent="0.4">
       <c r="A26" s="3" t="s">
         <v>11</v>
       </c>
@@ -3995,7 +4007,7 @@
       <c r="F26" s="3"/>
       <c r="G26" s="4"/>
     </row>
-    <row r="27" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:7" ht="41.65" x14ac:dyDescent="0.4">
       <c r="A27" s="3" t="s">
         <v>14</v>
       </c>
@@ -4012,7 +4024,7 @@
       <c r="F27" s="3"/>
       <c r="G27" s="4"/>
     </row>
-    <row r="28" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:7" ht="41.65" x14ac:dyDescent="0.4">
       <c r="A28" s="3" t="s">
         <v>17</v>
       </c>
@@ -4029,7 +4041,7 @@
       <c r="F28" s="3"/>
       <c r="G28" s="4"/>
     </row>
-    <row r="29" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:7" ht="55.5" x14ac:dyDescent="0.4">
       <c r="A29" s="3" t="s">
         <v>21</v>
       </c>
@@ -4046,7 +4058,7 @@
       <c r="F29" s="3"/>
       <c r="G29" s="4"/>
     </row>
-    <row r="30" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:7" ht="27.75" x14ac:dyDescent="0.4">
       <c r="A30" s="3" t="s">
         <v>25</v>
       </c>
@@ -4063,7 +4075,7 @@
       <c r="F30" s="3"/>
       <c r="G30" s="4"/>
     </row>
-    <row r="31" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:7" ht="41.65" x14ac:dyDescent="0.4">
       <c r="A31" s="3" t="s">
         <v>28</v>
       </c>
@@ -4080,7 +4092,7 @@
       <c r="F31" s="3"/>
       <c r="G31" s="4"/>
     </row>
-    <row r="32" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:7" ht="41.65" x14ac:dyDescent="0.4">
       <c r="A32" s="3" t="s">
         <v>31</v>
       </c>
@@ -4097,7 +4109,7 @@
       <c r="F32" s="3"/>
       <c r="G32" s="4"/>
     </row>
-    <row r="33" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:7" ht="55.5" x14ac:dyDescent="0.4">
       <c r="A33" s="3" t="s">
         <v>35</v>
       </c>
@@ -4114,7 +4126,7 @@
       <c r="F33" s="3"/>
       <c r="G33" s="4"/>
     </row>
-    <row r="34" spans="1:7" ht="116" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:7" ht="111" x14ac:dyDescent="0.4">
       <c r="A34" s="3" t="s">
         <v>36</v>
       </c>
@@ -4133,7 +4145,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="35" spans="1:7" ht="116" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:7" ht="111" x14ac:dyDescent="0.4">
       <c r="A35" s="3" t="s">
         <v>37</v>
       </c>
@@ -4152,7 +4164,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="36" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:7" ht="55.5" x14ac:dyDescent="0.4">
       <c r="A36" s="3" t="s">
         <v>38</v>
       </c>
@@ -4171,7 +4183,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="37" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:7" ht="55.5" x14ac:dyDescent="0.4">
       <c r="A37" s="3" t="s">
         <v>39</v>
       </c>
@@ -4190,7 +4202,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="38" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:7" ht="55.5" x14ac:dyDescent="0.4">
       <c r="A38" s="3" t="s">
         <v>162</v>
       </c>
@@ -4209,7 +4221,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="39" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:7" ht="55.5" x14ac:dyDescent="0.4">
       <c r="A39" s="3" t="s">
         <v>163</v>
       </c>
@@ -4228,7 +4240,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="40" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:7" ht="55.5" x14ac:dyDescent="0.4">
       <c r="A40" s="3" t="s">
         <v>40</v>
       </c>
@@ -4247,7 +4259,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="41" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:7" ht="55.5" x14ac:dyDescent="0.4">
       <c r="A41" s="3" t="s">
         <v>41</v>
       </c>
@@ -4266,7 +4278,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="42" spans="1:7" ht="87" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:7" ht="83.25" x14ac:dyDescent="0.4">
       <c r="A42" s="3" t="s">
         <v>42</v>
       </c>
@@ -4285,7 +4297,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="43" spans="1:7" ht="87" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:7" ht="83.25" x14ac:dyDescent="0.4">
       <c r="A43" s="3" t="s">
         <v>43</v>
       </c>
@@ -4304,7 +4316,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A44" s="3"/>
       <c r="B44" s="3"/>
       <c r="C44" s="3"/>
@@ -4313,7 +4325,7 @@
       <c r="F44" s="3"/>
       <c r="G44" s="4"/>
     </row>
-    <row r="45" spans="1:7" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:7" ht="83.25" x14ac:dyDescent="0.4">
       <c r="A45" s="9" t="s">
         <v>172</v>
       </c>
@@ -4336,7 +4348,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="46" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:7" ht="41.65" x14ac:dyDescent="0.4">
       <c r="A46" s="3" t="s">
         <v>10</v>
       </c>
@@ -4353,7 +4365,7 @@
       <c r="F46" s="3"/>
       <c r="G46" s="4"/>
     </row>
-    <row r="47" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:7" ht="27.75" x14ac:dyDescent="0.4">
       <c r="A47" s="3" t="s">
         <v>13</v>
       </c>
@@ -4370,7 +4382,7 @@
       <c r="F47" s="3"/>
       <c r="G47" s="4"/>
     </row>
-    <row r="48" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:7" ht="27.75" x14ac:dyDescent="0.4">
       <c r="A48" s="3" t="s">
         <v>16</v>
       </c>
@@ -4387,7 +4399,7 @@
       <c r="F48" s="3"/>
       <c r="G48" s="4"/>
     </row>
-    <row r="49" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:7" ht="27.75" x14ac:dyDescent="0.4">
       <c r="A49" s="3" t="s">
         <v>20</v>
       </c>
@@ -4404,7 +4416,7 @@
       <c r="F49" s="3"/>
       <c r="G49" s="4"/>
     </row>
-    <row r="50" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:7" ht="41.65" x14ac:dyDescent="0.4">
       <c r="A50" s="3" t="s">
         <v>24</v>
       </c>
@@ -4421,7 +4433,7 @@
       <c r="F50" s="3"/>
       <c r="G50" s="4"/>
     </row>
-    <row r="51" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:7" ht="27.75" x14ac:dyDescent="0.4">
       <c r="A51" s="3" t="s">
         <v>27</v>
       </c>
@@ -4438,7 +4450,7 @@
       <c r="F51" s="3"/>
       <c r="G51" s="4"/>
     </row>
-    <row r="52" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:7" ht="27.75" x14ac:dyDescent="0.4">
       <c r="A52" s="3" t="s">
         <v>30</v>
       </c>
@@ -4455,7 +4467,7 @@
       <c r="F52" s="3"/>
       <c r="G52" s="4"/>
     </row>
-    <row r="53" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:7" ht="27.75" x14ac:dyDescent="0.4">
       <c r="A53" s="3" t="s">
         <v>34</v>
       </c>
@@ -4472,7 +4484,7 @@
       <c r="F53" s="3"/>
       <c r="G53" s="4"/>
     </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A54" s="3"/>
       <c r="B54" s="3"/>
       <c r="C54" s="3"/>
@@ -4481,7 +4493,7 @@
       <c r="F54" s="3"/>
       <c r="G54" s="4"/>
     </row>
-    <row r="55" spans="1:7" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:7" ht="69.400000000000006" x14ac:dyDescent="0.4">
       <c r="A55" s="11" t="s">
         <v>173</v>
       </c>
@@ -4504,7 +4516,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A56" s="3" t="s">
         <v>44</v>
       </c>
@@ -4521,7 +4533,7 @@
       <c r="F56" s="3"/>
       <c r="G56" s="4"/>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A57" s="3" t="s">
         <v>45</v>
       </c>
@@ -4540,7 +4552,7 @@
       </c>
       <c r="G57" s="4"/>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A58" s="3" t="s">
         <v>46</v>
       </c>
@@ -4559,7 +4571,7 @@
       </c>
       <c r="G58" s="4"/>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A59" s="3" t="s">
         <v>47</v>
       </c>
@@ -4576,7 +4588,7 @@
       <c r="F59" s="3"/>
       <c r="G59" s="4"/>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A60" s="3" t="s">
         <v>48</v>
       </c>
@@ -4594,11 +4606,32 @@
       <c r="G60" s="4"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="6" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="e522a4ea-6824-496f-8ffe-e074cc291ac0">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="8080ce30-d5ea-40e8-a48f-b77958a33e4e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100CBEA71EDBDE86541B7589EDD610CDCA6" ma:contentTypeVersion="10" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="6135c02e9fba22fa14c95532ff73e585">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="e522a4ea-6824-496f-8ffe-e074cc291ac0" xmlns:ns3="8080ce30-d5ea-40e8-a48f-b77958a33e4e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4c9beda59bcc2e0dae0951e4601e1985" ns2:_="" ns3:_="">
     <xsd:import namespace="e522a4ea-6824-496f-8ffe-e074cc291ac0"/>
@@ -4789,27 +4822,32 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{13FE4927-61BE-41A1-B367-1B1C5D848E2B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="e522a4ea-6824-496f-8ffe-e074cc291ac0"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="8080ce30-d5ea-40e8-a48f-b77958a33e4e"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="e522a4ea-6824-496f-8ffe-e074cc291ac0">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="8080ce30-d5ea-40e8-a48f-b77958a33e4e" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8E8BB74B-0686-4136-81AA-6AA3532E32A8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EF3A5692-B908-4374-9724-9509DDA5EAF8}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -4826,29 +4864,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8E8BB74B-0686-4136-81AA-6AA3532E32A8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{13FE4927-61BE-41A1-B367-1B1C5D848E2B}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="e522a4ea-6824-496f-8ffe-e074cc291ac0"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="8080ce30-d5ea-40e8-a48f-b77958a33e4e"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>